<commit_message>
Adding KML files for download, corrections to data to fix obscure duplicate packet issue, and fixes to the pre- and post-flight data trimming
</commit_message>
<xml_diff>
--- a/www/flightdata/xlsx/flights_metadata.xlsx
+++ b/www/flightdata/xlsx/flights_metadata.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="814" uniqueCount="535">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="814" uniqueCount="534">
   <si>
     <t>flight</t>
   </si>
@@ -1087,7 +1087,7 @@
     <t>[{'transition': 'high_to_low', 'altitude_ft': 54081.0, 'altitude_m': 16483.89}]</t>
   </si>
   <si>
-    <t>[{'transition': 'low_to_high', 'altitude_ft': 5773.0, 'altitude_m': 1759.61}, {'transition': 'high_to_low', 'altitude_ft': 43536.0, 'altitude_m': 13269.77}]</t>
+    <t>[{'transition': 'high_to_low', 'altitude_ft': 43536.0, 'altitude_m': 13269.77}]</t>
   </si>
   <si>
     <t>[{'transition': 'high_to_low', 'altitude_ft': 45552.0, 'altitude_m': 13884.25}]</t>
@@ -1153,7 +1153,7 @@
     <t>[{'transition': 'high_to_low', 'altitude_ft': 68226.0, 'altitude_m': 20795.28}]</t>
   </si>
   <si>
-    <t>[{'transition': 'low_to_high', 'altitude_ft': 9581.0, 'altitude_m': 2920.29}, {'transition': 'high_to_low', 'altitude_ft': 55168.0, 'altitude_m': 16815.21}]</t>
+    <t>[{'transition': 'low_to_high', 'altitude_ft': 10274.0, 'altitude_m': 3131.52}, {'transition': 'high_to_low', 'altitude_ft': 55168.0, 'altitude_m': 16815.21}]</t>
   </si>
   <si>
     <t>[{'transition': 'low_to_high', 'altitude_ft': 16931.0, 'altitude_m': 5160.57}, {'transition': 'high_to_low', 'altitude_ft': 46196.0, 'altitude_m': 14080.54}]</t>
@@ -1180,7 +1180,7 @@
     <t>[{'transition': 'high_to_low', 'altitude_ft': 40575.0, 'altitude_m': 12367.26}]</t>
   </si>
   <si>
-    <t>[{'transition': 'low_to_high', 'altitude_ft': 5795.0, 'altitude_m': 1766.32}]</t>
+    <t>[{'transition': 'low_to_high', 'altitude_ft': 41108.0, 'altitude_m': 12529.72}]</t>
   </si>
   <si>
     <t>[{'transition': 'high_to_low', 'altitude_ft': 52066.0, 'altitude_m': 15869.72}]</t>
@@ -1213,7 +1213,7 @@
     <t>[{'transition': 'high_to_low', 'altitude_ft': 48301.0, 'altitude_m': 14722.14}]</t>
   </si>
   <si>
-    <t>[{'transition': 'low_to_high', 'altitude_ft': 9997.0, 'altitude_m': 3047.09}, {'transition': 'high_to_low', 'altitude_ft': 55507.0, 'altitude_m': 16918.53}]</t>
+    <t>[{'transition': 'high_to_low', 'altitude_ft': 55507.0, 'altitude_m': 16918.53}]</t>
   </si>
   <si>
     <t>[{'transition': 'high_to_low', 'altitude_ft': 54974.0, 'altitude_m': 16756.08}]</t>
@@ -1240,7 +1240,7 @@
     <t>[{'transition': 'high_to_low', 'altitude_ft': 52446.0, 'altitude_m': 15985.54}]</t>
   </si>
   <si>
-    <t>[{'transition': 'low_to_high', 'altitude_ft': 5949.0, 'altitude_m': 1813.26}, {'transition': 'high_to_low', 'altitude_ft': 62431.0, 'altitude_m': 19028.97}]</t>
+    <t>[{'transition': 'high_to_low', 'altitude_ft': 62431.0, 'altitude_m': 19028.97}]</t>
   </si>
   <si>
     <t>[{'transition': 'high_to_low', 'altitude_ft': 51806.0, 'altitude_m': 15790.47}]</t>
@@ -1252,7 +1252,7 @@
     <t>[{'transition': 'high_to_low', 'altitude_ft': 50361.0, 'altitude_m': 15350.03}]</t>
   </si>
   <si>
-    <t>[{'transition': 'low_to_high', 'altitude_ft': 7718.0, 'altitude_m': 2352.45}, {'transition': 'high_to_low', 'altitude_ft': 56579.0, 'altitude_m': 17245.28}]</t>
+    <t>[{'transition': 'high_to_low', 'altitude_ft': 56579.0, 'altitude_m': 17245.28}]</t>
   </si>
   <si>
     <t>[{'transition': 'high_to_low', 'altitude_ft': 48010.0, 'altitude_m': 14633.45}]</t>
@@ -1285,7 +1285,7 @@
     <t>[{'transition': 'high_to_low', 'altitude_ft': 53199.0, 'altitude_m': 16215.06}]</t>
   </si>
   <si>
-    <t>[{'transition': 'low_to_high', 'altitude_ft': 8118.0, 'altitude_m': 2474.37}, {'transition': 'high_to_low', 'altitude_ft': 55820.0, 'altitude_m': 17013.94}]</t>
+    <t>[{'transition': 'high_to_low', 'altitude_ft': 55820.0, 'altitude_m': 17013.94}]</t>
   </si>
   <si>
     <t>[{'transition': 'high_to_low', 'altitude_ft': 66320.0, 'altitude_m': 20214.34}]</t>
@@ -1297,7 +1297,7 @@
     <t>[{'transition': 'low_to_high', 'altitude_ft': 21272.0, 'altitude_m': 6483.71}, {'transition': 'high_to_low', 'altitude_ft': 74152.0, 'altitude_m': 22601.53}]</t>
   </si>
   <si>
-    <t>[{'transition': 'low_to_high', 'altitude_ft': 5667.0, 'altitude_m': 1727.3}, {'transition': 'high_to_low', 'altitude_ft': 40581.0, 'altitude_m': 12369.09}]</t>
+    <t>[{'transition': 'high_to_low', 'altitude_ft': 40581.0, 'altitude_m': 12369.09}]</t>
   </si>
   <si>
     <t>[{'transition': 'high_to_low', 'altitude_ft': 40592.0, 'altitude_m': 12372.44}]</t>
@@ -1309,7 +1309,7 @@
     <t>[{'transition': 'high_to_low', 'altitude_ft': 52415.0, 'altitude_m': 15976.09}]</t>
   </si>
   <si>
-    <t>[{'transition': 'low_to_high', 'altitude_ft': 8489.0, 'altitude_m': 2587.45}, {'transition': 'high_to_low', 'altitude_ft': 62268.0, 'altitude_m': 18979.29}]</t>
+    <t>[{'transition': 'high_to_low', 'altitude_ft': 62268.0, 'altitude_m': 18979.29}]</t>
   </si>
   <si>
     <t>[{'transition': 'low_to_high', 'altitude_ft': 12462.0, 'altitude_m': 3798.42}, {'transition': 'high_to_low', 'altitude_ft': 52124.0, 'altitude_m': 15887.4}]</t>
@@ -1327,7 +1327,7 @@
     <t>[{'transition': 'high_to_low', 'altitude_ft': 32694.0, 'altitude_m': 9965.13}]</t>
   </si>
   <si>
-    <t>[{'transition': 'low_to_high', 'altitude_ft': 9847.0, 'altitude_m': 3001.37}, {'transition': 'high_to_low', 'altitude_ft': 48953.0, 'altitude_m': 14920.87}]</t>
+    <t>[{'transition': 'low_to_high', 'altitude_ft': 10474.0, 'altitude_m': 3192.48}, {'transition': 'high_to_low', 'altitude_ft': 48953.0, 'altitude_m': 14920.87}]</t>
   </si>
   <si>
     <t>[{'transition': 'high_to_low', 'altitude_ft': 74746.0, 'altitude_m': 22782.58}]</t>
@@ -1363,7 +1363,7 @@
     <t>2hrs 19mins 53secs</t>
   </si>
   <si>
-    <t>2hrs 20mins 20secs</t>
+    <t>2hrs 28mins 20secs</t>
   </si>
   <si>
     <t>1hrs 38mins 0secs</t>
@@ -1375,7 +1375,7 @@
     <t>2hrs 27mins 30secs</t>
   </si>
   <si>
-    <t>1hrs 15mins 38secs</t>
+    <t>1hrs 24mins 38secs</t>
   </si>
   <si>
     <t>2hrs 8mins 20secs</t>
@@ -1393,7 +1393,7 @@
     <t>2hrs 4mins 47secs</t>
   </si>
   <si>
-    <t>1hrs 48mins 0secs</t>
+    <t>1hrs 51mins 0secs</t>
   </si>
   <si>
     <t>1hrs 57mins 30secs</t>
@@ -1411,7 +1411,7 @@
     <t>1hrs 55mins 0secs</t>
   </si>
   <si>
-    <t>1hrs 57mins 34secs</t>
+    <t>2hrs 6mins 4secs</t>
   </si>
   <si>
     <t>1hrs 26mins 40secs</t>
@@ -1453,7 +1453,7 @@
     <t>1hrs 31mins 20secs</t>
   </si>
   <si>
-    <t>1hrs 23mins 18secs</t>
+    <t>1hrs 33mins 18secs</t>
   </si>
   <si>
     <t>1hrs 42mins 48secs</t>
@@ -1468,7 +1468,7 @@
     <t>1hrs 52mins 0secs</t>
   </si>
   <si>
-    <t>2hrs 6mins 34secs</t>
+    <t>1hrs 39mins 4secs</t>
   </si>
   <si>
     <t>1hrs 50mins 26secs</t>
@@ -1531,9 +1531,6 @@
     <t>2hrs 1mins 12secs</t>
   </si>
   <si>
-    <t>1hrs 38mins 18secs</t>
-  </si>
-  <si>
     <t>1hrs 56mins 4secs</t>
   </si>
   <si>
@@ -1543,7 +1540,7 @@
     <t>2hrs 14mins 57secs</t>
   </si>
   <si>
-    <t>2hrs 7mins 48secs</t>
+    <t>2hrs 9mins 48secs</t>
   </si>
   <si>
     <t>1hrs 44mins 0secs</t>
@@ -1555,10 +1552,10 @@
     <t>2hrs 14mins 0secs</t>
   </si>
   <si>
-    <t>2hrs 12mins 0secs</t>
-  </si>
-  <si>
-    <t>2hrs 14mins 48secs</t>
+    <t>2hrs 13mins 30secs</t>
+  </si>
+  <si>
+    <t>2hrs 15mins 48secs</t>
   </si>
   <si>
     <t>1hrs 48mins 12secs</t>
@@ -1576,7 +1573,7 @@
     <t>1hrs 39mins 44secs</t>
   </si>
   <si>
-    <t>1hrs 53mins 30secs</t>
+    <t>1hrs 53mins 12secs</t>
   </si>
   <si>
     <t>2hrs 5mins 33secs</t>
@@ -1591,7 +1588,7 @@
     <t>1hrs 50mins 30secs</t>
   </si>
   <si>
-    <t>2hrs 36mins 30secs</t>
+    <t>2hrs 37mins 30secs</t>
   </si>
   <si>
     <t>0hrs 25mins 26secs</t>
@@ -1603,7 +1600,7 @@
     <t>2hrs 16mins 30secs</t>
   </si>
   <si>
-    <t>1hrs 58mins 33secs</t>
+    <t>1hrs 59mins 31secs</t>
   </si>
   <si>
     <t>2hrs 3mins 0secs</t>
@@ -2124,7 +2121,7 @@
         <v>27272.59</v>
       </c>
       <c r="J2">
-        <v>221</v>
+        <v>355</v>
       </c>
       <c r="K2" t="s">
         <v>443</v>
@@ -2240,7 +2237,7 @@
         <v>30445.86</v>
       </c>
       <c r="J3">
-        <v>350</v>
+        <v>543</v>
       </c>
       <c r="K3" t="s">
         <v>444</v>
@@ -2249,10 +2246,10 @@
         <v>5870</v>
       </c>
       <c r="M3">
-        <v>93.79000000000001</v>
+        <v>93.8</v>
       </c>
       <c r="N3">
-        <v>150.94</v>
+        <v>150.95</v>
       </c>
       <c r="O3">
         <v>7.8</v>
@@ -2297,16 +2294,16 @@
         <v>8.550000000000001</v>
       </c>
       <c r="AC3">
-        <v>40.2246666667</v>
+        <v>40.2248333333</v>
       </c>
       <c r="AD3">
         <v>-104.0771666667</v>
       </c>
       <c r="AE3">
-        <v>4567</v>
+        <v>4555</v>
       </c>
       <c r="AF3">
-        <v>1392.02</v>
+        <v>1388.36</v>
       </c>
       <c r="AG3">
         <v>39.4631666667</v>
@@ -2315,10 +2312,10 @@
         <v>-102.612</v>
       </c>
       <c r="AI3">
-        <v>93.79000000000001</v>
+        <v>93.8</v>
       </c>
       <c r="AJ3">
-        <v>150.94</v>
+        <v>150.95</v>
       </c>
       <c r="AK3">
         <v>5140</v>
@@ -2356,7 +2353,7 @@
         <v>29202.58</v>
       </c>
       <c r="J4">
-        <v>331</v>
+        <v>521</v>
       </c>
       <c r="K4" t="s">
         <v>445</v>
@@ -2472,7 +2469,7 @@
         <v>31019.5</v>
       </c>
       <c r="J5">
-        <v>333</v>
+        <v>599</v>
       </c>
       <c r="K5" t="s">
         <v>446</v>
@@ -2588,7 +2585,7 @@
         <v>29367.48</v>
       </c>
       <c r="J6">
-        <v>449</v>
+        <v>724</v>
       </c>
       <c r="K6" t="s">
         <v>447</v>
@@ -2704,7 +2701,7 @@
         <v>29403.45</v>
       </c>
       <c r="J7">
-        <v>542</v>
+        <v>822</v>
       </c>
       <c r="K7" t="s">
         <v>448</v>
@@ -2820,13 +2817,13 @@
         <v>28844.14</v>
       </c>
       <c r="J8">
-        <v>487</v>
+        <v>778</v>
       </c>
       <c r="K8" t="s">
         <v>449</v>
       </c>
       <c r="L8">
-        <v>8420</v>
+        <v>8900</v>
       </c>
       <c r="M8">
         <v>34.17</v>
@@ -2901,10 +2898,10 @@
         <v>54.99</v>
       </c>
       <c r="AK8">
-        <v>5106</v>
+        <v>5109</v>
       </c>
       <c r="AL8">
-        <v>1556.31</v>
+        <v>1557.22</v>
       </c>
     </row>
     <row r="9" spans="1:38">
@@ -2936,7 +2933,7 @@
         <v>29907.89</v>
       </c>
       <c r="J9">
-        <v>710</v>
+        <v>1088</v>
       </c>
       <c r="K9" t="s">
         <v>450</v>
@@ -2945,10 +2942,10 @@
         <v>5880</v>
       </c>
       <c r="M9">
-        <v>22.05</v>
+        <v>22.03</v>
       </c>
       <c r="N9">
-        <v>35.49</v>
+        <v>35.45</v>
       </c>
       <c r="O9">
         <v>9.59</v>
@@ -3005,22 +3002,22 @@
         <v>1742.54</v>
       </c>
       <c r="AG9">
-        <v>39.5968333333</v>
+        <v>39.5965</v>
       </c>
       <c r="AH9">
         <v>-103.462</v>
       </c>
       <c r="AI9">
-        <v>22.05</v>
+        <v>22.03</v>
       </c>
       <c r="AJ9">
-        <v>35.49</v>
+        <v>35.45</v>
       </c>
       <c r="AK9">
-        <v>5273</v>
+        <v>5271</v>
       </c>
       <c r="AL9">
-        <v>1607.21</v>
+        <v>1606.6</v>
       </c>
     </row>
     <row r="10" spans="1:38">
@@ -3052,7 +3049,7 @@
         <v>29527.2</v>
       </c>
       <c r="J10">
-        <v>571</v>
+        <v>896</v>
       </c>
       <c r="K10" t="s">
         <v>451</v>
@@ -3168,7 +3165,7 @@
         <v>27177.49</v>
       </c>
       <c r="J11">
-        <v>214</v>
+        <v>331</v>
       </c>
       <c r="K11" t="s">
         <v>452</v>
@@ -3284,13 +3281,13 @@
         <v>19231.97</v>
       </c>
       <c r="J12">
-        <v>434</v>
+        <v>671</v>
       </c>
       <c r="K12" t="s">
         <v>453</v>
       </c>
       <c r="L12">
-        <v>4538</v>
+        <v>5078</v>
       </c>
       <c r="M12">
         <v>15.88</v>
@@ -3365,10 +3362,10 @@
         <v>25.56</v>
       </c>
       <c r="AK12">
-        <v>5359</v>
+        <v>5360</v>
       </c>
       <c r="AL12">
-        <v>1633.42</v>
+        <v>1633.73</v>
       </c>
     </row>
     <row r="13" spans="1:38">
@@ -3400,7 +3397,7 @@
         <v>28522.27</v>
       </c>
       <c r="J13">
-        <v>456</v>
+        <v>720</v>
       </c>
       <c r="K13" t="s">
         <v>454</v>
@@ -3516,7 +3513,7 @@
         <v>26529.49</v>
       </c>
       <c r="J14">
-        <v>673</v>
+        <v>1023</v>
       </c>
       <c r="K14" t="s">
         <v>455</v>
@@ -3632,7 +3629,7 @@
         <v>27397.25</v>
       </c>
       <c r="J15">
-        <v>424</v>
+        <v>670</v>
       </c>
       <c r="K15" t="s">
         <v>456</v>
@@ -3748,7 +3745,7 @@
         <v>30407.76</v>
       </c>
       <c r="J16">
-        <v>444</v>
+        <v>679</v>
       </c>
       <c r="K16" t="s">
         <v>457</v>
@@ -3864,7 +3861,7 @@
         <v>27814.22</v>
       </c>
       <c r="J17">
-        <v>487</v>
+        <v>652</v>
       </c>
       <c r="K17" t="s">
         <v>458</v>
@@ -3980,13 +3977,13 @@
         <v>28673.76</v>
       </c>
       <c r="J18">
-        <v>620</v>
+        <v>954</v>
       </c>
       <c r="K18" t="s">
         <v>459</v>
       </c>
       <c r="L18">
-        <v>6480</v>
+        <v>6660</v>
       </c>
       <c r="M18">
         <v>25.8</v>
@@ -4061,10 +4058,10 @@
         <v>41.52</v>
       </c>
       <c r="AK18">
-        <v>6014</v>
+        <v>6017</v>
       </c>
       <c r="AL18">
-        <v>1833.07</v>
+        <v>1833.98</v>
       </c>
     </row>
     <row r="19" spans="1:38">
@@ -4096,7 +4093,7 @@
         <v>28635.66</v>
       </c>
       <c r="J19">
-        <v>695</v>
+        <v>969</v>
       </c>
       <c r="K19" t="s">
         <v>460</v>
@@ -4212,7 +4209,7 @@
         <v>29112.97</v>
       </c>
       <c r="J20">
-        <v>258</v>
+        <v>395</v>
       </c>
       <c r="K20" t="s">
         <v>461</v>
@@ -4328,7 +4325,7 @@
         <v>27902.61</v>
       </c>
       <c r="J21">
-        <v>503</v>
+        <v>765</v>
       </c>
       <c r="K21" t="s">
         <v>462</v>
@@ -4444,7 +4441,7 @@
         <v>27201.88</v>
       </c>
       <c r="J22">
-        <v>309</v>
+        <v>471</v>
       </c>
       <c r="K22" t="s">
         <v>463</v>
@@ -4560,7 +4557,7 @@
         <v>26864.16</v>
       </c>
       <c r="J23">
-        <v>375</v>
+        <v>586</v>
       </c>
       <c r="K23" t="s">
         <v>464</v>
@@ -4676,13 +4673,13 @@
         <v>27619.45</v>
       </c>
       <c r="J24">
-        <v>427</v>
+        <v>671</v>
       </c>
       <c r="K24" t="s">
         <v>465</v>
       </c>
       <c r="L24">
-        <v>7054</v>
+        <v>7564</v>
       </c>
       <c r="M24">
         <v>35.7</v>
@@ -4757,10 +4754,10 @@
         <v>57.46</v>
       </c>
       <c r="AK24">
-        <v>6055</v>
+        <v>6063</v>
       </c>
       <c r="AL24">
-        <v>1845.56</v>
+        <v>1848</v>
       </c>
     </row>
     <row r="25" spans="1:38">
@@ -4792,7 +4789,7 @@
         <v>25754.99</v>
       </c>
       <c r="J25">
-        <v>285</v>
+        <v>445</v>
       </c>
       <c r="K25" t="s">
         <v>466</v>
@@ -4908,7 +4905,7 @@
         <v>32334.71</v>
       </c>
       <c r="J26">
-        <v>488</v>
+        <v>745</v>
       </c>
       <c r="K26" t="s">
         <v>467</v>
@@ -5024,7 +5021,7 @@
         <v>30171.24</v>
       </c>
       <c r="J27">
-        <v>428</v>
+        <v>649</v>
       </c>
       <c r="K27" t="s">
         <v>468</v>
@@ -5140,7 +5137,7 @@
         <v>30216.65</v>
       </c>
       <c r="J28">
-        <v>494</v>
+        <v>750</v>
       </c>
       <c r="K28" t="s">
         <v>469</v>
@@ -5256,7 +5253,7 @@
         <v>30473.9</v>
       </c>
       <c r="J29">
-        <v>627</v>
+        <v>947</v>
       </c>
       <c r="K29" t="s">
         <v>470</v>
@@ -5372,7 +5369,7 @@
         <v>31062.47</v>
       </c>
       <c r="J30">
-        <v>527</v>
+        <v>807</v>
       </c>
       <c r="K30" t="s">
         <v>471</v>
@@ -5488,7 +5485,7 @@
         <v>27275.03</v>
       </c>
       <c r="J31">
-        <v>152</v>
+        <v>250</v>
       </c>
       <c r="K31" t="s">
         <v>472</v>
@@ -5604,7 +5601,7 @@
         <v>27295.45</v>
       </c>
       <c r="J32">
-        <v>226</v>
+        <v>282</v>
       </c>
       <c r="K32" t="s">
         <v>473</v>
@@ -5720,7 +5717,7 @@
         <v>27576.17</v>
       </c>
       <c r="J33">
-        <v>381</v>
+        <v>599</v>
       </c>
       <c r="K33" t="s">
         <v>474</v>
@@ -5836,7 +5833,7 @@
         <v>33452.41</v>
       </c>
       <c r="J34">
-        <v>479</v>
+        <v>731</v>
       </c>
       <c r="K34" t="s">
         <v>475</v>
@@ -5952,7 +5949,7 @@
         <v>30120.64</v>
       </c>
       <c r="J35">
-        <v>420</v>
+        <v>563</v>
       </c>
       <c r="K35" t="s">
         <v>476</v>
@@ -6068,7 +6065,7 @@
         <v>22073.92</v>
       </c>
       <c r="J36">
-        <v>282</v>
+        <v>435</v>
       </c>
       <c r="K36" t="s">
         <v>477</v>
@@ -6184,7 +6181,7 @@
         <v>22054.11</v>
       </c>
       <c r="J37">
-        <v>362</v>
+        <v>548</v>
       </c>
       <c r="K37" t="s">
         <v>478</v>
@@ -6300,13 +6297,13 @@
         <v>20454.52</v>
       </c>
       <c r="J38">
-        <v>295</v>
+        <v>416</v>
       </c>
       <c r="K38" t="s">
         <v>479</v>
       </c>
       <c r="L38">
-        <v>4998</v>
+        <v>5598</v>
       </c>
       <c r="M38">
         <v>40.85</v>
@@ -6381,10 +6378,10 @@
         <v>65.73999999999999</v>
       </c>
       <c r="AK38">
-        <v>4969</v>
+        <v>4965</v>
       </c>
       <c r="AL38">
-        <v>1514.55</v>
+        <v>1513.33</v>
       </c>
     </row>
     <row r="39" spans="1:38">
@@ -6416,7 +6413,7 @@
         <v>24134.98</v>
       </c>
       <c r="J39">
-        <v>388</v>
+        <v>524</v>
       </c>
       <c r="K39" t="s">
         <v>480</v>
@@ -6532,7 +6529,7 @@
         <v>30659.53</v>
       </c>
       <c r="J40">
-        <v>395</v>
+        <v>552</v>
       </c>
       <c r="K40" t="s">
         <v>481</v>
@@ -6648,7 +6645,7 @@
         <v>22799.95</v>
       </c>
       <c r="J41">
-        <v>486</v>
+        <v>686</v>
       </c>
       <c r="K41" t="s">
         <v>482</v>
@@ -6764,7 +6761,7 @@
         <v>26498.4</v>
       </c>
       <c r="J42">
-        <v>378</v>
+        <v>528</v>
       </c>
       <c r="K42" t="s">
         <v>483</v>
@@ -6880,7 +6877,7 @@
         <v>29330.6</v>
       </c>
       <c r="J43">
-        <v>376</v>
+        <v>564</v>
       </c>
       <c r="K43" t="s">
         <v>462</v>
@@ -6996,13 +6993,13 @@
         <v>31116.12</v>
       </c>
       <c r="J44">
-        <v>492</v>
+        <v>531</v>
       </c>
       <c r="K44" t="s">
         <v>484</v>
       </c>
       <c r="L44">
-        <v>7594</v>
+        <v>5944</v>
       </c>
       <c r="M44">
         <v>7.51</v>
@@ -7053,16 +7050,16 @@
         <v>8.25</v>
       </c>
       <c r="AC44">
-        <v>39.2362166667</v>
+        <v>39.2361333333</v>
       </c>
       <c r="AD44">
-        <v>-103.6967666667</v>
+        <v>-103.6969333333</v>
       </c>
       <c r="AE44">
-        <v>5362</v>
+        <v>5408</v>
       </c>
       <c r="AF44">
-        <v>1634.34</v>
+        <v>1648.36</v>
       </c>
       <c r="AG44">
         <v>39.1518333333</v>
@@ -7112,7 +7109,7 @@
         <v>31472.73</v>
       </c>
       <c r="J45">
-        <v>434</v>
+        <v>580</v>
       </c>
       <c r="K45" t="s">
         <v>485</v>
@@ -7228,7 +7225,7 @@
         <v>24002.7</v>
       </c>
       <c r="J46">
-        <v>195</v>
+        <v>322</v>
       </c>
       <c r="K46" t="s">
         <v>486</v>
@@ -7344,7 +7341,7 @@
         <v>30852.77</v>
       </c>
       <c r="J47">
-        <v>413</v>
+        <v>563</v>
       </c>
       <c r="K47" t="s">
         <v>487</v>
@@ -7460,7 +7457,7 @@
         <v>25859.54</v>
       </c>
       <c r="J48">
-        <v>427</v>
+        <v>601</v>
       </c>
       <c r="K48" t="s">
         <v>488</v>
@@ -7576,7 +7573,7 @@
         <v>28050.44</v>
       </c>
       <c r="J49">
-        <v>460</v>
+        <v>628</v>
       </c>
       <c r="K49" t="s">
         <v>489</v>
@@ -7692,7 +7689,7 @@
         <v>29633.57</v>
       </c>
       <c r="J50">
-        <v>506</v>
+        <v>687</v>
       </c>
       <c r="K50" t="s">
         <v>490</v>
@@ -7808,7 +7805,7 @@
         <v>32055.82</v>
       </c>
       <c r="J51">
-        <v>461</v>
+        <v>613</v>
       </c>
       <c r="K51" t="s">
         <v>491</v>
@@ -7924,7 +7921,7 @@
         <v>19250.56</v>
       </c>
       <c r="J52">
-        <v>329</v>
+        <v>454</v>
       </c>
       <c r="K52" t="s">
         <v>492</v>
@@ -8040,7 +8037,7 @@
         <v>32826.96</v>
       </c>
       <c r="J53">
-        <v>472</v>
+        <v>640</v>
       </c>
       <c r="K53" t="s">
         <v>493</v>
@@ -8156,7 +8153,7 @@
         <v>31589.17</v>
       </c>
       <c r="J54">
-        <v>384</v>
+        <v>525</v>
       </c>
       <c r="K54" t="s">
         <v>487</v>
@@ -8272,7 +8269,7 @@
         <v>26277.11</v>
       </c>
       <c r="J55">
-        <v>212</v>
+        <v>241</v>
       </c>
       <c r="K55" t="s">
         <v>494</v>
@@ -8388,7 +8385,7 @@
         <v>28106.52</v>
       </c>
       <c r="J56">
-        <v>367</v>
+        <v>512</v>
       </c>
       <c r="K56" t="s">
         <v>495</v>
@@ -8504,7 +8501,7 @@
         <v>29048.35</v>
       </c>
       <c r="J57">
-        <v>471</v>
+        <v>637</v>
       </c>
       <c r="K57" t="s">
         <v>489</v>
@@ -8620,7 +8617,7 @@
         <v>33886.75</v>
       </c>
       <c r="J58">
-        <v>573</v>
+        <v>813</v>
       </c>
       <c r="K58" t="s">
         <v>496</v>
@@ -8736,7 +8733,7 @@
         <v>31058.82</v>
       </c>
       <c r="J59">
-        <v>420</v>
+        <v>564</v>
       </c>
       <c r="K59" t="s">
         <v>497</v>
@@ -8852,7 +8849,7 @@
         <v>28350.06</v>
       </c>
       <c r="J60">
-        <v>677</v>
+        <v>950</v>
       </c>
       <c r="K60" t="s">
         <v>498</v>
@@ -8968,7 +8965,7 @@
         <v>26934.87</v>
       </c>
       <c r="J61">
-        <v>352</v>
+        <v>465</v>
       </c>
       <c r="K61" t="s">
         <v>499</v>
@@ -9084,7 +9081,7 @@
         <v>27902.61</v>
       </c>
       <c r="J62">
-        <v>480</v>
+        <v>678</v>
       </c>
       <c r="K62" t="s">
         <v>475</v>
@@ -9200,7 +9197,7 @@
         <v>28033.37</v>
       </c>
       <c r="J63">
-        <v>432</v>
+        <v>601</v>
       </c>
       <c r="K63" t="s">
         <v>500</v>
@@ -9316,7 +9313,7 @@
         <v>28398.22</v>
       </c>
       <c r="J64">
-        <v>493</v>
+        <v>662</v>
       </c>
       <c r="K64" t="s">
         <v>501</v>
@@ -9432,7 +9429,7 @@
         <v>28182.42</v>
       </c>
       <c r="J65">
-        <v>492</v>
+        <v>659</v>
       </c>
       <c r="K65" t="s">
         <v>502</v>
@@ -9548,7 +9545,7 @@
         <v>20625.82</v>
       </c>
       <c r="J66">
-        <v>337</v>
+        <v>457</v>
       </c>
       <c r="K66" t="s">
         <v>503</v>
@@ -9664,7 +9661,7 @@
         <v>28004.41</v>
       </c>
       <c r="J67">
-        <v>429</v>
+        <v>593</v>
       </c>
       <c r="K67" t="s">
         <v>504</v>
@@ -9780,19 +9777,19 @@
         <v>28943.5</v>
       </c>
       <c r="J68">
-        <v>567</v>
+        <v>794</v>
       </c>
       <c r="K68" t="s">
-        <v>505</v>
+        <v>450</v>
       </c>
       <c r="L68">
-        <v>5898</v>
+        <v>5880</v>
       </c>
       <c r="M68">
-        <v>39.34</v>
+        <v>39.31</v>
       </c>
       <c r="N68">
-        <v>63.3</v>
+        <v>63.26</v>
       </c>
       <c r="O68">
         <v>14.77</v>
@@ -9837,34 +9834,34 @@
         <v>11.81</v>
       </c>
       <c r="AC68">
-        <v>39.6085</v>
+        <v>39.6081666667</v>
       </c>
       <c r="AD68">
-        <v>-104.04235</v>
+        <v>-104.0421666667</v>
       </c>
       <c r="AE68">
-        <v>5217</v>
+        <v>5211</v>
       </c>
       <c r="AF68">
-        <v>1590.14</v>
+        <v>1588.31</v>
       </c>
       <c r="AG68">
-        <v>39.2631666667</v>
+        <v>39.2631833333</v>
       </c>
       <c r="AH68">
-        <v>-103.4556666667</v>
+        <v>-103.4557666667</v>
       </c>
       <c r="AI68">
-        <v>39.34</v>
+        <v>39.31</v>
       </c>
       <c r="AJ68">
-        <v>63.3</v>
+        <v>63.26</v>
       </c>
       <c r="AK68">
-        <v>8248</v>
+        <v>8278</v>
       </c>
       <c r="AL68">
-        <v>2513.99</v>
+        <v>2523.13</v>
       </c>
     </row>
     <row r="69" spans="1:38">
@@ -9896,10 +9893,10 @@
         <v>28393.64</v>
       </c>
       <c r="J69">
-        <v>436</v>
+        <v>594</v>
       </c>
       <c r="K69" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="L69">
         <v>6964</v>
@@ -10012,10 +10009,10 @@
         <v>29202.89</v>
       </c>
       <c r="J70">
-        <v>451</v>
+        <v>609</v>
       </c>
       <c r="K70" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
       <c r="L70">
         <v>6990</v>
@@ -10128,10 +10125,10 @@
         <v>32300.27</v>
       </c>
       <c r="J71">
+        <v>695</v>
+      </c>
+      <c r="K71" t="s">
         <v>507</v>
-      </c>
-      <c r="K71" t="s">
-        <v>508</v>
       </c>
       <c r="L71">
         <v>8097</v>
@@ -10244,13 +10241,13 @@
         <v>29960.62</v>
       </c>
       <c r="J72">
-        <v>733</v>
+        <v>1042</v>
       </c>
       <c r="K72" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="L72">
-        <v>7668</v>
+        <v>7788</v>
       </c>
       <c r="M72">
         <v>41.87</v>
@@ -10325,10 +10322,10 @@
         <v>67.38</v>
       </c>
       <c r="AK72">
-        <v>4697</v>
+        <v>4699</v>
       </c>
       <c r="AL72">
-        <v>1431.65</v>
+        <v>1432.26</v>
       </c>
     </row>
     <row r="73" spans="1:38">
@@ -10360,10 +10357,10 @@
         <v>33012.89</v>
       </c>
       <c r="J73">
-        <v>377</v>
+        <v>515</v>
       </c>
       <c r="K73" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="L73">
         <v>6240</v>
@@ -10476,10 +10473,10 @@
         <v>28324.45</v>
       </c>
       <c r="J74">
-        <v>431</v>
+        <v>580</v>
       </c>
       <c r="K74" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="L74">
         <v>6882</v>
@@ -10592,10 +10589,10 @@
         <v>29625.95</v>
       </c>
       <c r="J75">
-        <v>505</v>
+        <v>679</v>
       </c>
       <c r="K75" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="L75">
         <v>8040</v>
@@ -10708,13 +10705,13 @@
         <v>30095.34</v>
       </c>
       <c r="J76">
-        <v>336</v>
+        <v>622</v>
       </c>
       <c r="K76" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="L76">
-        <v>7920</v>
+        <v>8010</v>
       </c>
       <c r="M76">
         <v>21.98</v>
@@ -10824,13 +10821,13 @@
         <v>30091.68</v>
       </c>
       <c r="J77">
-        <v>464</v>
+        <v>640</v>
       </c>
       <c r="K77" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
       <c r="L77">
-        <v>8088</v>
+        <v>8148</v>
       </c>
       <c r="M77">
         <v>22.83</v>
@@ -10905,10 +10902,10 @@
         <v>36.75</v>
       </c>
       <c r="AK77">
-        <v>5392</v>
+        <v>5390</v>
       </c>
       <c r="AL77">
-        <v>1643.48</v>
+        <v>1642.87</v>
       </c>
     </row>
     <row r="78" spans="1:38">
@@ -10940,10 +10937,10 @@
         <v>28709.72</v>
       </c>
       <c r="J78">
-        <v>414</v>
+        <v>559</v>
       </c>
       <c r="K78" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="L78">
         <v>6492</v>
@@ -11056,10 +11053,10 @@
         <v>32196.94</v>
       </c>
       <c r="J79">
-        <v>205</v>
+        <v>235</v>
       </c>
       <c r="K79" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="L79">
         <v>7638</v>
@@ -11172,10 +11169,10 @@
         <v>30373.62</v>
       </c>
       <c r="J80">
-        <v>425</v>
+        <v>573</v>
       </c>
       <c r="K80" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="L80">
         <v>6750</v>
@@ -11288,10 +11285,10 @@
         <v>29959.1</v>
       </c>
       <c r="J81">
-        <v>209</v>
+        <v>246</v>
       </c>
       <c r="K81" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="L81">
         <v>5718</v>
@@ -11404,10 +11401,10 @@
         <v>31915</v>
       </c>
       <c r="J82">
-        <v>721</v>
+        <v>979</v>
       </c>
       <c r="K82" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="L82">
         <v>5984</v>
@@ -11520,19 +11517,19 @@
         <v>27361.9</v>
       </c>
       <c r="J83">
-        <v>482</v>
+        <v>665</v>
       </c>
       <c r="K83" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="L83">
-        <v>6810</v>
+        <v>6792</v>
       </c>
       <c r="M83">
-        <v>58.13</v>
+        <v>58.16</v>
       </c>
       <c r="N83">
-        <v>93.55</v>
+        <v>93.59</v>
       </c>
       <c r="O83">
         <v>6.7</v>
@@ -11577,16 +11574,16 @@
         <v>8.01</v>
       </c>
       <c r="AC83">
-        <v>39.6075</v>
+        <v>39.6078333333</v>
       </c>
       <c r="AD83">
-        <v>-104.0411166667</v>
+        <v>-104.0413333333</v>
       </c>
       <c r="AE83">
-        <v>5220</v>
+        <v>5218</v>
       </c>
       <c r="AF83">
-        <v>1591.06</v>
+        <v>1590.45</v>
       </c>
       <c r="AG83">
         <v>38.87505</v>
@@ -11595,10 +11592,10 @@
         <v>-103.50505</v>
       </c>
       <c r="AI83">
-        <v>58.13</v>
+        <v>58.16</v>
       </c>
       <c r="AJ83">
-        <v>93.55</v>
+        <v>93.59</v>
       </c>
       <c r="AK83">
         <v>5473</v>
@@ -11636,10 +11633,10 @@
         <v>27325.62</v>
       </c>
       <c r="J84">
-        <v>435</v>
+        <v>594</v>
       </c>
       <c r="K84" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="L84">
         <v>7533</v>
@@ -11752,10 +11749,10 @@
         <v>27549.65</v>
       </c>
       <c r="J85">
-        <v>512</v>
+        <v>696</v>
       </c>
       <c r="K85" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="L85">
         <v>8396</v>
@@ -11868,10 +11865,10 @@
         <v>30593.39</v>
       </c>
       <c r="J86">
-        <v>626</v>
+        <v>894</v>
       </c>
       <c r="K86" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="L86">
         <v>7043</v>
@@ -11984,10 +11981,10 @@
         <v>33555.43</v>
       </c>
       <c r="J87">
-        <v>425</v>
+        <v>569</v>
       </c>
       <c r="K87" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="L87">
         <v>6630</v>
@@ -12100,13 +12097,13 @@
         <v>30007.86</v>
       </c>
       <c r="J88">
-        <v>864</v>
+        <v>1234</v>
       </c>
       <c r="K88" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="L88">
-        <v>9390</v>
+        <v>9450</v>
       </c>
       <c r="M88">
         <v>55.17</v>
@@ -12181,10 +12178,10 @@
         <v>88.78</v>
       </c>
       <c r="AK88">
-        <v>6135</v>
+        <v>6144</v>
       </c>
       <c r="AL88">
-        <v>1869.95</v>
+        <v>1872.69</v>
       </c>
     </row>
     <row r="89" spans="1:38">
@@ -12216,10 +12213,10 @@
         <v>3420.77</v>
       </c>
       <c r="J89">
-        <v>95</v>
+        <v>127</v>
       </c>
       <c r="K89" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="L89">
         <v>1526</v>
@@ -12332,10 +12329,10 @@
         <v>28377.49</v>
       </c>
       <c r="J90">
-        <v>400</v>
+        <v>538</v>
       </c>
       <c r="K90" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="L90">
         <v>6300</v>
@@ -12448,10 +12445,10 @@
         <v>25712.32</v>
       </c>
       <c r="J91">
-        <v>452</v>
+        <v>651</v>
       </c>
       <c r="K91" t="s">
-        <v>528</v>
+        <v>527</v>
       </c>
       <c r="L91">
         <v>8190</v>
@@ -12564,13 +12561,13 @@
         <v>26009.19</v>
       </c>
       <c r="J92">
-        <v>227</v>
+        <v>386</v>
       </c>
       <c r="K92" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="L92">
-        <v>7113</v>
+        <v>7171</v>
       </c>
       <c r="M92">
         <v>109.11</v>
@@ -12680,10 +12677,10 @@
         <v>31706.21</v>
       </c>
       <c r="J93">
-        <v>474</v>
+        <v>632</v>
       </c>
       <c r="K93" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="L93">
         <v>7380</v>
@@ -12796,10 +12793,10 @@
         <v>33558.78</v>
       </c>
       <c r="J94">
-        <v>357</v>
+        <v>515</v>
       </c>
       <c r="K94" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="L94">
         <v>7830</v>
@@ -12912,10 +12909,10 @@
         <v>27113.79</v>
       </c>
       <c r="J95">
-        <v>365</v>
+        <v>499</v>
       </c>
       <c r="K95" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="L95">
         <v>6495</v>
@@ -13028,10 +13025,10 @@
         <v>28232.1</v>
       </c>
       <c r="J96">
-        <v>487</v>
+        <v>650</v>
       </c>
       <c r="K96" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="L96">
         <v>7830</v>
@@ -13144,10 +13141,10 @@
         <v>32628.84</v>
       </c>
       <c r="J97">
-        <v>784</v>
+        <v>1017</v>
       </c>
       <c r="K97" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="L97">
         <v>8910</v>
@@ -13260,10 +13257,10 @@
         <v>31353.86</v>
       </c>
       <c r="J98">
-        <v>500</v>
+        <v>669</v>
       </c>
       <c r="K98" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="L98">
         <v>7695</v>

</xml_diff>

<commit_message>
Accidentally left status packets interleaved with position packets
</commit_message>
<xml_diff>
--- a/www/flightdata/xlsx/flights_metadata.xlsx
+++ b/www/flightdata/xlsx/flights_metadata.xlsx
@@ -2121,7 +2121,7 @@
         <v>27272.59</v>
       </c>
       <c r="J2">
-        <v>355</v>
+        <v>221</v>
       </c>
       <c r="K2" t="s">
         <v>443</v>
@@ -2237,7 +2237,7 @@
         <v>30445.86</v>
       </c>
       <c r="J3">
-        <v>543</v>
+        <v>350</v>
       </c>
       <c r="K3" t="s">
         <v>444</v>
@@ -2353,7 +2353,7 @@
         <v>29202.58</v>
       </c>
       <c r="J4">
-        <v>521</v>
+        <v>331</v>
       </c>
       <c r="K4" t="s">
         <v>445</v>
@@ -2469,7 +2469,7 @@
         <v>31019.5</v>
       </c>
       <c r="J5">
-        <v>599</v>
+        <v>333</v>
       </c>
       <c r="K5" t="s">
         <v>446</v>
@@ -2585,7 +2585,7 @@
         <v>29367.48</v>
       </c>
       <c r="J6">
-        <v>724</v>
+        <v>449</v>
       </c>
       <c r="K6" t="s">
         <v>447</v>
@@ -2701,7 +2701,7 @@
         <v>29403.45</v>
       </c>
       <c r="J7">
-        <v>822</v>
+        <v>542</v>
       </c>
       <c r="K7" t="s">
         <v>448</v>
@@ -2817,7 +2817,7 @@
         <v>28844.14</v>
       </c>
       <c r="J8">
-        <v>778</v>
+        <v>492</v>
       </c>
       <c r="K8" t="s">
         <v>449</v>
@@ -2933,7 +2933,7 @@
         <v>29907.89</v>
       </c>
       <c r="J9">
-        <v>1088</v>
+        <v>709</v>
       </c>
       <c r="K9" t="s">
         <v>450</v>
@@ -3049,7 +3049,7 @@
         <v>29527.2</v>
       </c>
       <c r="J10">
-        <v>896</v>
+        <v>571</v>
       </c>
       <c r="K10" t="s">
         <v>451</v>
@@ -3165,7 +3165,7 @@
         <v>27177.49</v>
       </c>
       <c r="J11">
-        <v>331</v>
+        <v>214</v>
       </c>
       <c r="K11" t="s">
         <v>452</v>
@@ -3281,7 +3281,7 @@
         <v>19231.97</v>
       </c>
       <c r="J12">
-        <v>671</v>
+        <v>439</v>
       </c>
       <c r="K12" t="s">
         <v>453</v>
@@ -3397,7 +3397,7 @@
         <v>28522.27</v>
       </c>
       <c r="J13">
-        <v>720</v>
+        <v>456</v>
       </c>
       <c r="K13" t="s">
         <v>454</v>
@@ -3513,7 +3513,7 @@
         <v>26529.49</v>
       </c>
       <c r="J14">
-        <v>1023</v>
+        <v>673</v>
       </c>
       <c r="K14" t="s">
         <v>455</v>
@@ -3629,7 +3629,7 @@
         <v>27397.25</v>
       </c>
       <c r="J15">
-        <v>670</v>
+        <v>424</v>
       </c>
       <c r="K15" t="s">
         <v>456</v>
@@ -3745,7 +3745,7 @@
         <v>30407.76</v>
       </c>
       <c r="J16">
-        <v>679</v>
+        <v>444</v>
       </c>
       <c r="K16" t="s">
         <v>457</v>
@@ -3861,7 +3861,7 @@
         <v>27814.22</v>
       </c>
       <c r="J17">
-        <v>652</v>
+        <v>487</v>
       </c>
       <c r="K17" t="s">
         <v>458</v>
@@ -3977,7 +3977,7 @@
         <v>28673.76</v>
       </c>
       <c r="J18">
-        <v>954</v>
+        <v>623</v>
       </c>
       <c r="K18" t="s">
         <v>459</v>
@@ -4093,7 +4093,7 @@
         <v>28635.66</v>
       </c>
       <c r="J19">
-        <v>969</v>
+        <v>695</v>
       </c>
       <c r="K19" t="s">
         <v>460</v>
@@ -4209,7 +4209,7 @@
         <v>29112.97</v>
       </c>
       <c r="J20">
-        <v>395</v>
+        <v>258</v>
       </c>
       <c r="K20" t="s">
         <v>461</v>
@@ -4325,7 +4325,7 @@
         <v>27902.61</v>
       </c>
       <c r="J21">
-        <v>765</v>
+        <v>503</v>
       </c>
       <c r="K21" t="s">
         <v>462</v>
@@ -4441,7 +4441,7 @@
         <v>27201.88</v>
       </c>
       <c r="J22">
-        <v>471</v>
+        <v>309</v>
       </c>
       <c r="K22" t="s">
         <v>463</v>
@@ -4557,7 +4557,7 @@
         <v>26864.16</v>
       </c>
       <c r="J23">
-        <v>586</v>
+        <v>375</v>
       </c>
       <c r="K23" t="s">
         <v>464</v>
@@ -4673,7 +4673,7 @@
         <v>27619.45</v>
       </c>
       <c r="J24">
-        <v>671</v>
+        <v>432</v>
       </c>
       <c r="K24" t="s">
         <v>465</v>
@@ -4789,7 +4789,7 @@
         <v>25754.99</v>
       </c>
       <c r="J25">
-        <v>445</v>
+        <v>285</v>
       </c>
       <c r="K25" t="s">
         <v>466</v>
@@ -4905,7 +4905,7 @@
         <v>32334.71</v>
       </c>
       <c r="J26">
-        <v>745</v>
+        <v>488</v>
       </c>
       <c r="K26" t="s">
         <v>467</v>
@@ -5021,7 +5021,7 @@
         <v>30171.24</v>
       </c>
       <c r="J27">
-        <v>649</v>
+        <v>428</v>
       </c>
       <c r="K27" t="s">
         <v>468</v>
@@ -5137,7 +5137,7 @@
         <v>30216.65</v>
       </c>
       <c r="J28">
-        <v>750</v>
+        <v>494</v>
       </c>
       <c r="K28" t="s">
         <v>469</v>
@@ -5253,7 +5253,7 @@
         <v>30473.9</v>
       </c>
       <c r="J29">
-        <v>947</v>
+        <v>627</v>
       </c>
       <c r="K29" t="s">
         <v>470</v>
@@ -5369,7 +5369,7 @@
         <v>31062.47</v>
       </c>
       <c r="J30">
-        <v>807</v>
+        <v>526</v>
       </c>
       <c r="K30" t="s">
         <v>471</v>
@@ -5485,7 +5485,7 @@
         <v>27275.03</v>
       </c>
       <c r="J31">
-        <v>250</v>
+        <v>152</v>
       </c>
       <c r="K31" t="s">
         <v>472</v>
@@ -5601,7 +5601,7 @@
         <v>27295.45</v>
       </c>
       <c r="J32">
-        <v>282</v>
+        <v>226</v>
       </c>
       <c r="K32" t="s">
         <v>473</v>
@@ -5717,7 +5717,7 @@
         <v>27576.17</v>
       </c>
       <c r="J33">
-        <v>599</v>
+        <v>381</v>
       </c>
       <c r="K33" t="s">
         <v>474</v>
@@ -5833,7 +5833,7 @@
         <v>33452.41</v>
       </c>
       <c r="J34">
-        <v>731</v>
+        <v>479</v>
       </c>
       <c r="K34" t="s">
         <v>475</v>
@@ -5949,7 +5949,7 @@
         <v>30120.64</v>
       </c>
       <c r="J35">
-        <v>563</v>
+        <v>420</v>
       </c>
       <c r="K35" t="s">
         <v>476</v>
@@ -6065,7 +6065,7 @@
         <v>22073.92</v>
       </c>
       <c r="J36">
-        <v>435</v>
+        <v>282</v>
       </c>
       <c r="K36" t="s">
         <v>477</v>
@@ -6181,7 +6181,7 @@
         <v>22054.11</v>
       </c>
       <c r="J37">
-        <v>548</v>
+        <v>362</v>
       </c>
       <c r="K37" t="s">
         <v>478</v>
@@ -6297,7 +6297,7 @@
         <v>20454.52</v>
       </c>
       <c r="J38">
-        <v>416</v>
+        <v>302</v>
       </c>
       <c r="K38" t="s">
         <v>479</v>
@@ -6413,7 +6413,7 @@
         <v>24134.98</v>
       </c>
       <c r="J39">
-        <v>524</v>
+        <v>388</v>
       </c>
       <c r="K39" t="s">
         <v>480</v>
@@ -6529,7 +6529,7 @@
         <v>30659.53</v>
       </c>
       <c r="J40">
-        <v>552</v>
+        <v>395</v>
       </c>
       <c r="K40" t="s">
         <v>481</v>
@@ -6645,7 +6645,7 @@
         <v>22799.95</v>
       </c>
       <c r="J41">
-        <v>686</v>
+        <v>486</v>
       </c>
       <c r="K41" t="s">
         <v>482</v>
@@ -6761,7 +6761,7 @@
         <v>26498.4</v>
       </c>
       <c r="J42">
-        <v>528</v>
+        <v>378</v>
       </c>
       <c r="K42" t="s">
         <v>483</v>
@@ -6877,7 +6877,7 @@
         <v>29330.6</v>
       </c>
       <c r="J43">
-        <v>564</v>
+        <v>376</v>
       </c>
       <c r="K43" t="s">
         <v>462</v>
@@ -6993,7 +6993,7 @@
         <v>31116.12</v>
       </c>
       <c r="J44">
-        <v>531</v>
+        <v>392</v>
       </c>
       <c r="K44" t="s">
         <v>484</v>
@@ -7109,7 +7109,7 @@
         <v>31472.73</v>
       </c>
       <c r="J45">
-        <v>580</v>
+        <v>434</v>
       </c>
       <c r="K45" t="s">
         <v>485</v>
@@ -7225,7 +7225,7 @@
         <v>24002.7</v>
       </c>
       <c r="J46">
-        <v>322</v>
+        <v>195</v>
       </c>
       <c r="K46" t="s">
         <v>486</v>
@@ -7341,7 +7341,7 @@
         <v>30852.77</v>
       </c>
       <c r="J47">
-        <v>563</v>
+        <v>413</v>
       </c>
       <c r="K47" t="s">
         <v>487</v>
@@ -7457,7 +7457,7 @@
         <v>25859.54</v>
       </c>
       <c r="J48">
-        <v>601</v>
+        <v>427</v>
       </c>
       <c r="K48" t="s">
         <v>488</v>
@@ -7573,7 +7573,7 @@
         <v>28050.44</v>
       </c>
       <c r="J49">
-        <v>628</v>
+        <v>460</v>
       </c>
       <c r="K49" t="s">
         <v>489</v>
@@ -7689,7 +7689,7 @@
         <v>29633.57</v>
       </c>
       <c r="J50">
-        <v>687</v>
+        <v>506</v>
       </c>
       <c r="K50" t="s">
         <v>490</v>
@@ -7805,7 +7805,7 @@
         <v>32055.82</v>
       </c>
       <c r="J51">
-        <v>613</v>
+        <v>461</v>
       </c>
       <c r="K51" t="s">
         <v>491</v>
@@ -7921,7 +7921,7 @@
         <v>19250.56</v>
       </c>
       <c r="J52">
-        <v>454</v>
+        <v>329</v>
       </c>
       <c r="K52" t="s">
         <v>492</v>
@@ -8037,7 +8037,7 @@
         <v>32826.96</v>
       </c>
       <c r="J53">
-        <v>640</v>
+        <v>472</v>
       </c>
       <c r="K53" t="s">
         <v>493</v>
@@ -8153,7 +8153,7 @@
         <v>31589.17</v>
       </c>
       <c r="J54">
-        <v>525</v>
+        <v>384</v>
       </c>
       <c r="K54" t="s">
         <v>487</v>
@@ -8269,7 +8269,7 @@
         <v>26277.11</v>
       </c>
       <c r="J55">
-        <v>241</v>
+        <v>212</v>
       </c>
       <c r="K55" t="s">
         <v>494</v>
@@ -8385,7 +8385,7 @@
         <v>28106.52</v>
       </c>
       <c r="J56">
-        <v>512</v>
+        <v>367</v>
       </c>
       <c r="K56" t="s">
         <v>495</v>
@@ -8501,7 +8501,7 @@
         <v>29048.35</v>
       </c>
       <c r="J57">
-        <v>637</v>
+        <v>471</v>
       </c>
       <c r="K57" t="s">
         <v>489</v>
@@ -8617,7 +8617,7 @@
         <v>33886.75</v>
       </c>
       <c r="J58">
-        <v>813</v>
+        <v>573</v>
       </c>
       <c r="K58" t="s">
         <v>496</v>
@@ -8733,7 +8733,7 @@
         <v>31058.82</v>
       </c>
       <c r="J59">
-        <v>564</v>
+        <v>420</v>
       </c>
       <c r="K59" t="s">
         <v>497</v>
@@ -8849,7 +8849,7 @@
         <v>28350.06</v>
       </c>
       <c r="J60">
-        <v>950</v>
+        <v>677</v>
       </c>
       <c r="K60" t="s">
         <v>498</v>
@@ -8965,7 +8965,7 @@
         <v>26934.87</v>
       </c>
       <c r="J61">
-        <v>465</v>
+        <v>352</v>
       </c>
       <c r="K61" t="s">
         <v>499</v>
@@ -9081,7 +9081,7 @@
         <v>27902.61</v>
       </c>
       <c r="J62">
-        <v>678</v>
+        <v>480</v>
       </c>
       <c r="K62" t="s">
         <v>475</v>
@@ -9197,7 +9197,7 @@
         <v>28033.37</v>
       </c>
       <c r="J63">
-        <v>601</v>
+        <v>432</v>
       </c>
       <c r="K63" t="s">
         <v>500</v>
@@ -9313,7 +9313,7 @@
         <v>28398.22</v>
       </c>
       <c r="J64">
-        <v>662</v>
+        <v>493</v>
       </c>
       <c r="K64" t="s">
         <v>501</v>
@@ -9429,7 +9429,7 @@
         <v>28182.42</v>
       </c>
       <c r="J65">
-        <v>659</v>
+        <v>492</v>
       </c>
       <c r="K65" t="s">
         <v>502</v>
@@ -9545,7 +9545,7 @@
         <v>20625.82</v>
       </c>
       <c r="J66">
-        <v>457</v>
+        <v>337</v>
       </c>
       <c r="K66" t="s">
         <v>503</v>
@@ -9661,7 +9661,7 @@
         <v>28004.41</v>
       </c>
       <c r="J67">
-        <v>593</v>
+        <v>429</v>
       </c>
       <c r="K67" t="s">
         <v>504</v>
@@ -9777,7 +9777,7 @@
         <v>28943.5</v>
       </c>
       <c r="J68">
-        <v>794</v>
+        <v>566</v>
       </c>
       <c r="K68" t="s">
         <v>450</v>
@@ -9893,7 +9893,7 @@
         <v>28393.64</v>
       </c>
       <c r="J69">
-        <v>594</v>
+        <v>436</v>
       </c>
       <c r="K69" t="s">
         <v>505</v>
@@ -10009,7 +10009,7 @@
         <v>29202.89</v>
       </c>
       <c r="J70">
-        <v>609</v>
+        <v>451</v>
       </c>
       <c r="K70" t="s">
         <v>506</v>
@@ -10125,7 +10125,7 @@
         <v>32300.27</v>
       </c>
       <c r="J71">
-        <v>695</v>
+        <v>507</v>
       </c>
       <c r="K71" t="s">
         <v>507</v>
@@ -10241,7 +10241,7 @@
         <v>29960.62</v>
       </c>
       <c r="J72">
-        <v>1042</v>
+        <v>736</v>
       </c>
       <c r="K72" t="s">
         <v>508</v>
@@ -10357,7 +10357,7 @@
         <v>33012.89</v>
       </c>
       <c r="J73">
-        <v>515</v>
+        <v>377</v>
       </c>
       <c r="K73" t="s">
         <v>509</v>
@@ -10473,7 +10473,7 @@
         <v>28324.45</v>
       </c>
       <c r="J74">
-        <v>580</v>
+        <v>431</v>
       </c>
       <c r="K74" t="s">
         <v>510</v>
@@ -10589,7 +10589,7 @@
         <v>29625.95</v>
       </c>
       <c r="J75">
-        <v>679</v>
+        <v>505</v>
       </c>
       <c r="K75" t="s">
         <v>511</v>
@@ -10705,7 +10705,7 @@
         <v>30095.34</v>
       </c>
       <c r="J76">
-        <v>622</v>
+        <v>337</v>
       </c>
       <c r="K76" t="s">
         <v>512</v>
@@ -10821,7 +10821,7 @@
         <v>30091.68</v>
       </c>
       <c r="J77">
-        <v>640</v>
+        <v>465</v>
       </c>
       <c r="K77" t="s">
         <v>513</v>
@@ -10937,7 +10937,7 @@
         <v>28709.72</v>
       </c>
       <c r="J78">
-        <v>559</v>
+        <v>414</v>
       </c>
       <c r="K78" t="s">
         <v>514</v>
@@ -11053,7 +11053,7 @@
         <v>32196.94</v>
       </c>
       <c r="J79">
-        <v>235</v>
+        <v>205</v>
       </c>
       <c r="K79" t="s">
         <v>515</v>
@@ -11169,7 +11169,7 @@
         <v>30373.62</v>
       </c>
       <c r="J80">
-        <v>573</v>
+        <v>425</v>
       </c>
       <c r="K80" t="s">
         <v>516</v>
@@ -11285,7 +11285,7 @@
         <v>29959.1</v>
       </c>
       <c r="J81">
-        <v>246</v>
+        <v>209</v>
       </c>
       <c r="K81" t="s">
         <v>517</v>
@@ -11401,7 +11401,7 @@
         <v>31915</v>
       </c>
       <c r="J82">
-        <v>979</v>
+        <v>721</v>
       </c>
       <c r="K82" t="s">
         <v>518</v>
@@ -11517,7 +11517,7 @@
         <v>27361.9</v>
       </c>
       <c r="J83">
-        <v>665</v>
+        <v>481</v>
       </c>
       <c r="K83" t="s">
         <v>519</v>
@@ -11633,7 +11633,7 @@
         <v>27325.62</v>
       </c>
       <c r="J84">
-        <v>594</v>
+        <v>435</v>
       </c>
       <c r="K84" t="s">
         <v>520</v>
@@ -11749,7 +11749,7 @@
         <v>27549.65</v>
       </c>
       <c r="J85">
-        <v>696</v>
+        <v>512</v>
       </c>
       <c r="K85" t="s">
         <v>521</v>
@@ -11865,7 +11865,7 @@
         <v>30593.39</v>
       </c>
       <c r="J86">
-        <v>894</v>
+        <v>626</v>
       </c>
       <c r="K86" t="s">
         <v>522</v>
@@ -11981,7 +11981,7 @@
         <v>33555.43</v>
       </c>
       <c r="J87">
-        <v>569</v>
+        <v>425</v>
       </c>
       <c r="K87" t="s">
         <v>523</v>
@@ -12097,7 +12097,7 @@
         <v>30007.86</v>
       </c>
       <c r="J88">
-        <v>1234</v>
+        <v>866</v>
       </c>
       <c r="K88" t="s">
         <v>524</v>
@@ -12213,7 +12213,7 @@
         <v>3420.77</v>
       </c>
       <c r="J89">
-        <v>127</v>
+        <v>95</v>
       </c>
       <c r="K89" t="s">
         <v>525</v>
@@ -12329,7 +12329,7 @@
         <v>28377.49</v>
       </c>
       <c r="J90">
-        <v>538</v>
+        <v>400</v>
       </c>
       <c r="K90" t="s">
         <v>526</v>
@@ -12445,7 +12445,7 @@
         <v>25712.32</v>
       </c>
       <c r="J91">
-        <v>651</v>
+        <v>452</v>
       </c>
       <c r="K91" t="s">
         <v>527</v>
@@ -12561,7 +12561,7 @@
         <v>26009.19</v>
       </c>
       <c r="J92">
-        <v>386</v>
+        <v>229</v>
       </c>
       <c r="K92" t="s">
         <v>528</v>
@@ -12677,7 +12677,7 @@
         <v>31706.21</v>
       </c>
       <c r="J93">
-        <v>632</v>
+        <v>474</v>
       </c>
       <c r="K93" t="s">
         <v>529</v>
@@ -12793,7 +12793,7 @@
         <v>33558.78</v>
       </c>
       <c r="J94">
-        <v>515</v>
+        <v>357</v>
       </c>
       <c r="K94" t="s">
         <v>530</v>
@@ -12909,7 +12909,7 @@
         <v>27113.79</v>
       </c>
       <c r="J95">
-        <v>499</v>
+        <v>365</v>
       </c>
       <c r="K95" t="s">
         <v>531</v>
@@ -13025,7 +13025,7 @@
         <v>28232.1</v>
       </c>
       <c r="J96">
-        <v>650</v>
+        <v>487</v>
       </c>
       <c r="K96" t="s">
         <v>530</v>
@@ -13141,7 +13141,7 @@
         <v>32628.84</v>
       </c>
       <c r="J97">
-        <v>1017</v>
+        <v>784</v>
       </c>
       <c r="K97" t="s">
         <v>532</v>
@@ -13257,7 +13257,7 @@
         <v>31353.86</v>
       </c>
       <c r="J98">
-        <v>669</v>
+        <v>500</v>
       </c>
       <c r="K98" t="s">
         <v>533</v>

</xml_diff>

<commit_message>
Update to the EOSS-391 flight data to correct errors
</commit_message>
<xml_diff>
--- a/www/flightdata/xlsx/flights_metadata.xlsx
+++ b/www/flightdata/xlsx/flights_metadata.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="955" uniqueCount="560">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="955" uniqueCount="561">
   <si>
     <t>balloonsize</t>
   </si>
@@ -460,7 +460,7 @@
     <t>EOSS-307</t>
   </si>
   <si>
-    <t>1hrs 39mins 56secs</t>
+    <t>1hrs 39mins 44secs</t>
   </si>
   <si>
     <t>372</t>
@@ -1625,6 +1625,9 @@
   </si>
   <si>
     <t>EOSS-386</t>
+  </si>
+  <si>
+    <t>1hrs 37mins 50secs</t>
   </si>
   <si>
     <t>344</t>
@@ -3466,10 +3469,10 @@
         <v>1483.16</v>
       </c>
       <c r="M11">
-        <v>6.98</v>
+        <v>6.95</v>
       </c>
       <c r="N11">
-        <v>4.34</v>
+        <v>4.32</v>
       </c>
       <c r="O11">
         <v>40.606516666666664</v>
@@ -3478,16 +3481,16 @@
         <v>-104.32368333333334</v>
       </c>
       <c r="Q11">
-        <v>4973</v>
+        <v>4995</v>
       </c>
       <c r="R11">
-        <v>1515.77</v>
+        <v>1522.48</v>
       </c>
       <c r="S11">
-        <v>40.64908333333334</v>
+        <v>40.648833333333336</v>
       </c>
       <c r="T11">
-        <v>-104.3845</v>
+        <v>-104.38433333333332</v>
       </c>
       <c r="U11" t="s">
         <v>68</v>
@@ -3517,10 +3520,10 @@
         <v>1.63</v>
       </c>
       <c r="AD11">
-        <v>6.98</v>
+        <v>6.95</v>
       </c>
       <c r="AE11">
-        <v>4.34</v>
+        <v>4.32</v>
       </c>
       <c r="AF11" t="s">
         <v>107</v>
@@ -3639,7 +3642,7 @@
         <v>30007.86</v>
       </c>
       <c r="X12">
-        <v>865</v>
+        <v>864</v>
       </c>
       <c r="Y12" t="s">
         <v>53</v>
@@ -4434,7 +4437,7 @@
         <v>148</v>
       </c>
       <c r="I18">
-        <v>5996</v>
+        <v>5984</v>
       </c>
       <c r="J18" t="s">
         <v>149</v>
@@ -4458,16 +4461,16 @@
         <v>-103.01071666666668</v>
       </c>
       <c r="Q18">
-        <v>5235</v>
+        <v>5257</v>
       </c>
       <c r="R18">
-        <v>1595.63</v>
+        <v>1602.33</v>
       </c>
       <c r="S18">
-        <v>39.6085</v>
+        <v>39.60848333333333</v>
       </c>
       <c r="T18">
-        <v>-104.0405</v>
+        <v>-104.04043333333334</v>
       </c>
       <c r="U18" t="s">
         <v>60</v>
@@ -4479,7 +4482,7 @@
         <v>31915</v>
       </c>
       <c r="X18">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="Y18" t="s">
         <v>53</v>
@@ -15491,40 +15494,40 @@
         <v>536</v>
       </c>
       <c r="H97" t="s">
-        <v>218</v>
+        <v>537</v>
       </c>
       <c r="I97">
-        <v>5880</v>
+        <v>5870</v>
       </c>
       <c r="J97" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="K97">
-        <v>5066</v>
+        <v>5140</v>
       </c>
       <c r="L97">
-        <v>1544.12</v>
+        <v>1566.67</v>
       </c>
       <c r="M97">
-        <v>151</v>
+        <v>150.94</v>
       </c>
       <c r="N97">
-        <v>93.83</v>
+        <v>93.79</v>
       </c>
       <c r="O97">
-        <v>39.46233333333333</v>
+        <v>39.463166666666666</v>
       </c>
       <c r="P97">
         <v>-102.612</v>
       </c>
       <c r="Q97">
-        <v>4555</v>
+        <v>4567</v>
       </c>
       <c r="R97">
-        <v>1388.36</v>
+        <v>1392.02</v>
       </c>
       <c r="S97">
-        <v>40.224833333333336</v>
+        <v>40.224666666666664</v>
       </c>
       <c r="T97">
         <v>-104.07716666666668</v>
@@ -15539,7 +15542,7 @@
         <v>30445.86</v>
       </c>
       <c r="X97">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="Y97" t="s">
         <v>53</v>
@@ -15557,13 +15560,13 @@
         <v>1.7</v>
       </c>
       <c r="AD97">
-        <v>151</v>
+        <v>150.94</v>
       </c>
       <c r="AE97">
-        <v>93.83</v>
+        <v>93.79</v>
       </c>
       <c r="AF97" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="AG97">
         <v>3</v>
@@ -15628,16 +15631,16 @@
         <v>1</v>
       </c>
       <c r="G98" t="s">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="H98" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="I98">
         <v>5827</v>
       </c>
       <c r="J98" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="K98">
         <v>4606</v>
@@ -15703,7 +15706,7 @@
         <v>101.65</v>
       </c>
       <c r="AF98" t="s">
-        <v>541</v>
+        <v>542</v>
       </c>
       <c r="AG98">
         <v>3</v>
@@ -15753,10 +15756,10 @@
         <v>62</v>
       </c>
       <c r="B99" t="s">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="C99" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="D99">
         <v>76670</v>
@@ -15768,7 +15771,7 @@
         <v>1</v>
       </c>
       <c r="G99" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="H99" t="s">
         <v>160</v>
@@ -15777,7 +15780,7 @@
         <v>6750</v>
       </c>
       <c r="J99" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="K99">
         <v>5967</v>
@@ -15843,7 +15846,7 @@
         <v>112.5</v>
       </c>
       <c r="AF99" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
       <c r="AG99">
         <v>1.5</v>
@@ -15893,10 +15896,10 @@
         <v>62</v>
       </c>
       <c r="B100" t="s">
-        <v>547</v>
+        <v>548</v>
       </c>
       <c r="C100" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="D100">
         <v>91765</v>
@@ -15908,10 +15911,10 @@
         <v>1</v>
       </c>
       <c r="G100" t="s">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="H100" t="s">
-        <v>549</v>
+        <v>550</v>
       </c>
       <c r="I100">
         <v>7500</v>
@@ -15983,7 +15986,7 @@
         <v>109.03</v>
       </c>
       <c r="AF100" t="s">
-        <v>550</v>
+        <v>551</v>
       </c>
       <c r="AG100">
         <v>1.5</v>
@@ -16033,10 +16036,10 @@
         <v>62</v>
       </c>
       <c r="B101" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="C101" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="D101">
         <v>94256</v>
@@ -16048,10 +16051,10 @@
         <v>1</v>
       </c>
       <c r="G101" t="s">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="H101" t="s">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="I101">
         <v>7559</v>
@@ -16123,7 +16126,7 @@
         <v>106.3</v>
       </c>
       <c r="AF101" t="s">
-        <v>554</v>
+        <v>555</v>
       </c>
       <c r="AG101">
         <v>1.5</v>
@@ -16173,10 +16176,10 @@
         <v>62</v>
       </c>
       <c r="B102" t="s">
-        <v>555</v>
+        <v>556</v>
       </c>
       <c r="C102" t="s">
-        <v>556</v>
+        <v>557</v>
       </c>
       <c r="D102">
         <v>91900</v>
@@ -16188,10 +16191,10 @@
         <v>1</v>
       </c>
       <c r="G102" t="s">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="H102" t="s">
-        <v>558</v>
+        <v>559</v>
       </c>
       <c r="I102">
         <v>6922</v>
@@ -16263,7 +16266,7 @@
         <v>41.83</v>
       </c>
       <c r="AF102" t="s">
-        <v>559</v>
+        <v>560</v>
       </c>
       <c r="AG102">
         <v>1.5</v>

</xml_diff>

<commit_message>
Flight data for EOSS-392 and EOSS-392
</commit_message>
<xml_diff>
--- a/www/flightdata/xlsx/flights_metadata.xlsx
+++ b/www/flightdata/xlsx/flights_metadata.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="955" uniqueCount="561">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="973" uniqueCount="571">
   <si>
     <t>balloonsize</t>
   </si>
@@ -1697,6 +1697,36 @@
   </si>
   <si>
     <t>[{"altitude_ft":61585.0,"altitude_m":18771.11,"transition":"high_to_low"}]</t>
+  </si>
+  <si>
+    <t>2026-04-04</t>
+  </si>
+  <si>
+    <t>EOSS-392</t>
+  </si>
+  <si>
+    <t>1hrs 38mins 1secs</t>
+  </si>
+  <si>
+    <t>371</t>
+  </si>
+  <si>
+    <t>[{"altitude_ft":58392.0,"altitude_m":17797.88,"transition":"high_to_low"}]</t>
+  </si>
+  <si>
+    <t>["AE0SS-1","AE0SS-3"]</t>
+  </si>
+  <si>
+    <t>EOSS-393</t>
+  </si>
+  <si>
+    <t>2hrs 0mins 30secs</t>
+  </si>
+  <si>
+    <t>374</t>
+  </si>
+  <si>
+    <t>[{"altitude_ft":62992.0,"altitude_m":19199.96,"transition":"high_to_low"}]</t>
   </si>
 </sst>
 </file>
@@ -2028,7 +2058,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AT102"/>
+  <dimension ref="A1:AT104"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:46">
@@ -16311,6 +16341,286 @@
         <v>1.7</v>
       </c>
     </row>
+    <row r="103" spans="1:46">
+      <c r="A103" t="s">
+        <v>46</v>
+      </c>
+      <c r="B103" t="s">
+        <v>552</v>
+      </c>
+      <c r="C103" t="s">
+        <v>561</v>
+      </c>
+      <c r="D103">
+        <v>84489</v>
+      </c>
+      <c r="E103">
+        <v>25752.25</v>
+      </c>
+      <c r="F103" t="b">
+        <v>1</v>
+      </c>
+      <c r="G103" t="s">
+        <v>562</v>
+      </c>
+      <c r="H103" t="s">
+        <v>563</v>
+      </c>
+      <c r="I103">
+        <v>5881</v>
+      </c>
+      <c r="J103" t="s">
+        <v>564</v>
+      </c>
+      <c r="K103">
+        <v>5794</v>
+      </c>
+      <c r="L103">
+        <v>1766.01</v>
+      </c>
+      <c r="M103">
+        <v>83.62</v>
+      </c>
+      <c r="N103">
+        <v>51.96</v>
+      </c>
+      <c r="O103">
+        <v>39.25783333333333</v>
+      </c>
+      <c r="P103">
+        <v>-103.17983333333332</v>
+      </c>
+      <c r="Q103">
+        <v>5210</v>
+      </c>
+      <c r="R103">
+        <v>1588.01</v>
+      </c>
+      <c r="S103">
+        <v>39.60816666666667</v>
+      </c>
+      <c r="T103">
+        <v>-104.04216666666666</v>
+      </c>
+      <c r="U103" t="s">
+        <v>156</v>
+      </c>
+      <c r="V103">
+        <v>84283</v>
+      </c>
+      <c r="W103">
+        <v>25689.46</v>
+      </c>
+      <c r="X103">
+        <v>241</v>
+      </c>
+      <c r="Y103" t="s">
+        <v>53</v>
+      </c>
+      <c r="Z103">
+        <v>12</v>
+      </c>
+      <c r="AA103">
+        <v>3.66</v>
+      </c>
+      <c r="AB103">
+        <v>0.77</v>
+      </c>
+      <c r="AC103">
+        <v>1.7</v>
+      </c>
+      <c r="AD103">
+        <v>83.62</v>
+      </c>
+      <c r="AE103">
+        <v>51.96</v>
+      </c>
+      <c r="AF103" t="s">
+        <v>565</v>
+      </c>
+      <c r="AG103">
+        <v>3</v>
+      </c>
+      <c r="AH103">
+        <v>6.61</v>
+      </c>
+      <c r="AI103">
+        <v>5.07</v>
+      </c>
+      <c r="AJ103">
+        <v>11.18</v>
+      </c>
+      <c r="AK103">
+        <v>1.53</v>
+      </c>
+      <c r="AL103">
+        <v>3.38</v>
+      </c>
+      <c r="AM103">
+        <v>10.37</v>
+      </c>
+      <c r="AN103">
+        <v>22.86</v>
+      </c>
+      <c r="AO103">
+        <v>9.44</v>
+      </c>
+      <c r="AP103">
+        <v>20.82</v>
+      </c>
+      <c r="AQ103">
+        <v>7.37</v>
+      </c>
+      <c r="AR103">
+        <v>16.25</v>
+      </c>
+      <c r="AS103">
+        <v>0.77</v>
+      </c>
+      <c r="AT103">
+        <v>1.7</v>
+      </c>
+    </row>
+    <row r="104" spans="1:46">
+      <c r="A104" t="s">
+        <v>46</v>
+      </c>
+      <c r="B104" t="s">
+        <v>566</v>
+      </c>
+      <c r="C104" t="s">
+        <v>561</v>
+      </c>
+      <c r="D104">
+        <v>97827</v>
+      </c>
+      <c r="E104">
+        <v>29817.67</v>
+      </c>
+      <c r="F104" t="b">
+        <v>1</v>
+      </c>
+      <c r="G104" t="s">
+        <v>567</v>
+      </c>
+      <c r="H104" t="s">
+        <v>568</v>
+      </c>
+      <c r="I104">
+        <v>7230</v>
+      </c>
+      <c r="J104" t="s">
+        <v>569</v>
+      </c>
+      <c r="K104">
+        <v>4885</v>
+      </c>
+      <c r="L104">
+        <v>1488.95</v>
+      </c>
+      <c r="M104">
+        <v>96.51</v>
+      </c>
+      <c r="N104">
+        <v>59.97</v>
+      </c>
+      <c r="O104">
+        <v>39.25083333333333</v>
+      </c>
+      <c r="P104">
+        <v>-103.01733333333334</v>
+      </c>
+      <c r="Q104">
+        <v>5214</v>
+      </c>
+      <c r="R104">
+        <v>1589.23</v>
+      </c>
+      <c r="S104">
+        <v>39.60816666666667</v>
+      </c>
+      <c r="T104">
+        <v>-104.04233333333332</v>
+      </c>
+      <c r="U104" t="s">
+        <v>156</v>
+      </c>
+      <c r="V104">
+        <v>97827</v>
+      </c>
+      <c r="W104">
+        <v>29817.67</v>
+      </c>
+      <c r="X104">
+        <v>456</v>
+      </c>
+      <c r="Y104" t="s">
+        <v>53</v>
+      </c>
+      <c r="Z104">
+        <v>12</v>
+      </c>
+      <c r="AA104">
+        <v>3.66</v>
+      </c>
+      <c r="AB104">
+        <v>0.79</v>
+      </c>
+      <c r="AC104">
+        <v>1.75</v>
+      </c>
+      <c r="AD104">
+        <v>96.51</v>
+      </c>
+      <c r="AE104">
+        <v>59.97</v>
+      </c>
+      <c r="AF104" t="s">
+        <v>570</v>
+      </c>
+      <c r="AG104">
+        <v>3</v>
+      </c>
+      <c r="AH104">
+        <v>6.61</v>
+      </c>
+      <c r="AI104">
+        <v>5.2</v>
+      </c>
+      <c r="AJ104">
+        <v>11.47</v>
+      </c>
+      <c r="AK104">
+        <v>1.46</v>
+      </c>
+      <c r="AL104">
+        <v>3.21</v>
+      </c>
+      <c r="AM104">
+        <v>10.45</v>
+      </c>
+      <c r="AN104">
+        <v>23.04</v>
+      </c>
+      <c r="AO104">
+        <v>9.54</v>
+      </c>
+      <c r="AP104">
+        <v>21.04</v>
+      </c>
+      <c r="AQ104">
+        <v>7.45</v>
+      </c>
+      <c r="AR104">
+        <v>16.43</v>
+      </c>
+      <c r="AS104">
+        <v>0.79</v>
+      </c>
+      <c r="AT104">
+        <v>1.75</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Updates for historical data for EOSS-394 and EOSS-395
</commit_message>
<xml_diff>
--- a/www/flightdata/xlsx/flights_metadata.xlsx
+++ b/www/flightdata/xlsx/flights_metadata.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="973" uniqueCount="571">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="991" uniqueCount="579">
   <si>
     <t>balloonsize</t>
   </si>
@@ -1727,6 +1727,30 @@
   </si>
   <si>
     <t>[{"altitude_ft":62992.0,"altitude_m":19199.96,"transition":"high_to_low"}]</t>
+  </si>
+  <si>
+    <t>2026-04-12</t>
+  </si>
+  <si>
+    <t>EOSS-394</t>
+  </si>
+  <si>
+    <t>2hrs 7mins 30secs</t>
+  </si>
+  <si>
+    <t>[{"altitude_ft":41952.0,"altitude_m":12786.97,"transition":"high_to_low"},{"altitude_ft":54733.0,"altitude_m":16682.62,"transition":"low_to_high"}]</t>
+  </si>
+  <si>
+    <t>["KC0D-2","K0SCC-13","AE0SS-4"]</t>
+  </si>
+  <si>
+    <t>EOSS-395</t>
+  </si>
+  <si>
+    <t>1hrs 55mins 29secs</t>
+  </si>
+  <si>
+    <t>[{"altitude_ft":12263.0,"altitude_m":3737.76,"transition":"low_to_high"},{"altitude_ft":64144.0,"altitude_m":19551.09,"transition":"high_to_low"}]</t>
   </si>
 </sst>
 </file>
@@ -2058,7 +2082,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AT104"/>
+  <dimension ref="A1:AT106"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:46">
@@ -16621,6 +16645,286 @@
         <v>1.75</v>
       </c>
     </row>
+    <row r="105" spans="1:46">
+      <c r="A105" t="s">
+        <v>62</v>
+      </c>
+      <c r="B105" t="s">
+        <v>566</v>
+      </c>
+      <c r="C105" t="s">
+        <v>571</v>
+      </c>
+      <c r="D105">
+        <v>91837</v>
+      </c>
+      <c r="E105">
+        <v>27991.92</v>
+      </c>
+      <c r="F105" t="b">
+        <v>1</v>
+      </c>
+      <c r="G105" t="s">
+        <v>572</v>
+      </c>
+      <c r="H105" t="s">
+        <v>573</v>
+      </c>
+      <c r="I105">
+        <v>7650</v>
+      </c>
+      <c r="J105" t="s">
+        <v>372</v>
+      </c>
+      <c r="K105">
+        <v>4595</v>
+      </c>
+      <c r="L105">
+        <v>1400.56</v>
+      </c>
+      <c r="M105">
+        <v>90.57</v>
+      </c>
+      <c r="N105">
+        <v>56.28</v>
+      </c>
+      <c r="O105">
+        <v>40.01166666666666</v>
+      </c>
+      <c r="P105">
+        <v>-103.12033333333332</v>
+      </c>
+      <c r="Q105">
+        <v>5216</v>
+      </c>
+      <c r="R105">
+        <v>1589.84</v>
+      </c>
+      <c r="S105">
+        <v>39.608</v>
+      </c>
+      <c r="T105">
+        <v>-104.04216666666666</v>
+      </c>
+      <c r="U105" t="s">
+        <v>118</v>
+      </c>
+      <c r="V105">
+        <v>91612</v>
+      </c>
+      <c r="W105">
+        <v>27923.34</v>
+      </c>
+      <c r="X105">
+        <v>302</v>
+      </c>
+      <c r="Y105" t="s">
+        <v>53</v>
+      </c>
+      <c r="Z105">
+        <v>12</v>
+      </c>
+      <c r="AA105">
+        <v>3.66</v>
+      </c>
+      <c r="AB105">
+        <v>0.79</v>
+      </c>
+      <c r="AC105">
+        <v>1.75</v>
+      </c>
+      <c r="AD105">
+        <v>90.57</v>
+      </c>
+      <c r="AE105">
+        <v>56.28</v>
+      </c>
+      <c r="AF105" t="s">
+        <v>574</v>
+      </c>
+      <c r="AG105">
+        <v>1.5</v>
+      </c>
+      <c r="AH105">
+        <v>3.31</v>
+      </c>
+      <c r="AI105">
+        <v>3.46</v>
+      </c>
+      <c r="AJ105">
+        <v>7.62</v>
+      </c>
+      <c r="AK105">
+        <v>1.65</v>
+      </c>
+      <c r="AL105">
+        <v>3.64</v>
+      </c>
+      <c r="AM105">
+        <v>7.4</v>
+      </c>
+      <c r="AN105">
+        <v>16.32</v>
+      </c>
+      <c r="AO105">
+        <v>8.12</v>
+      </c>
+      <c r="AP105">
+        <v>17.91</v>
+      </c>
+      <c r="AQ105">
+        <v>5.9</v>
+      </c>
+      <c r="AR105">
+        <v>13.01</v>
+      </c>
+      <c r="AS105">
+        <v>0.79</v>
+      </c>
+      <c r="AT105">
+        <v>1.75</v>
+      </c>
+    </row>
+    <row r="106" spans="1:46">
+      <c r="A106" t="s">
+        <v>46</v>
+      </c>
+      <c r="B106" t="s">
+        <v>575</v>
+      </c>
+      <c r="C106" t="s">
+        <v>571</v>
+      </c>
+      <c r="D106">
+        <v>99167</v>
+      </c>
+      <c r="E106">
+        <v>30226.1</v>
+      </c>
+      <c r="F106" t="b">
+        <v>1</v>
+      </c>
+      <c r="G106" t="s">
+        <v>576</v>
+      </c>
+      <c r="H106" t="s">
+        <v>577</v>
+      </c>
+      <c r="I106">
+        <v>6929</v>
+      </c>
+      <c r="J106" t="s">
+        <v>263</v>
+      </c>
+      <c r="K106">
+        <v>4617</v>
+      </c>
+      <c r="L106">
+        <v>1407.26</v>
+      </c>
+      <c r="M106">
+        <v>85.13</v>
+      </c>
+      <c r="N106">
+        <v>52.9</v>
+      </c>
+      <c r="O106">
+        <v>39.89648333333333</v>
+      </c>
+      <c r="P106">
+        <v>-103.11896666666668</v>
+      </c>
+      <c r="Q106">
+        <v>5211</v>
+      </c>
+      <c r="R106">
+        <v>1588.31</v>
+      </c>
+      <c r="S106">
+        <v>39.608</v>
+      </c>
+      <c r="T106">
+        <v>-104.04216666666666</v>
+      </c>
+      <c r="U106" t="s">
+        <v>156</v>
+      </c>
+      <c r="V106">
+        <v>99059</v>
+      </c>
+      <c r="W106">
+        <v>30193.18</v>
+      </c>
+      <c r="X106">
+        <v>353</v>
+      </c>
+      <c r="Y106" t="s">
+        <v>53</v>
+      </c>
+      <c r="Z106">
+        <v>12</v>
+      </c>
+      <c r="AA106">
+        <v>3.66</v>
+      </c>
+      <c r="AB106">
+        <v>0.77</v>
+      </c>
+      <c r="AC106">
+        <v>1.7</v>
+      </c>
+      <c r="AD106">
+        <v>85.13</v>
+      </c>
+      <c r="AE106">
+        <v>52.9</v>
+      </c>
+      <c r="AF106" t="s">
+        <v>578</v>
+      </c>
+      <c r="AG106">
+        <v>3</v>
+      </c>
+      <c r="AH106">
+        <v>6.61</v>
+      </c>
+      <c r="AI106">
+        <v>7.02</v>
+      </c>
+      <c r="AJ106">
+        <v>15.47</v>
+      </c>
+      <c r="AK106">
+        <v>2.08</v>
+      </c>
+      <c r="AL106">
+        <v>4.58</v>
+      </c>
+      <c r="AM106">
+        <v>12.86</v>
+      </c>
+      <c r="AN106">
+        <v>28.36</v>
+      </c>
+      <c r="AO106">
+        <v>12.44</v>
+      </c>
+      <c r="AP106">
+        <v>27.42</v>
+      </c>
+      <c r="AQ106">
+        <v>9.87</v>
+      </c>
+      <c r="AR106">
+        <v>21.75</v>
+      </c>
+      <c r="AS106">
+        <v>0.77</v>
+      </c>
+      <c r="AT106">
+        <v>1.7</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Updates for flights EOSS-396 & EOSS-397
</commit_message>
<xml_diff>
--- a/www/flightdata/xlsx/flights_metadata.xlsx
+++ b/www/flightdata/xlsx/flights_metadata.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="991" uniqueCount="579">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1009" uniqueCount="588">
   <si>
     <t>balloonsize</t>
   </si>
@@ -1751,6 +1751,33 @@
   </si>
   <si>
     <t>[{"altitude_ft":12263.0,"altitude_m":3737.76,"transition":"low_to_high"},{"altitude_ft":64144.0,"altitude_m":19551.09,"transition":"high_to_low"}]</t>
+  </si>
+  <si>
+    <t>2026-04-19</t>
+  </si>
+  <si>
+    <t>EOSS-396</t>
+  </si>
+  <si>
+    <t>359</t>
+  </si>
+  <si>
+    <t>[{"altitude_ft":37233.0,"altitude_m":11348.62,"transition":"high_to_low"}]</t>
+  </si>
+  <si>
+    <t>["AE0SS-1","K0SCC-13","AE0SS-3"]</t>
+  </si>
+  <si>
+    <t>EOSS-397</t>
+  </si>
+  <si>
+    <t>2hrs 19mins 30secs</t>
+  </si>
+  <si>
+    <t>396</t>
+  </si>
+  <si>
+    <t>[{"altitude_ft":36584.0,"altitude_m":11150.8,"transition":"high_to_low"}]</t>
   </si>
 </sst>
 </file>
@@ -2082,7 +2109,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AT106"/>
+  <dimension ref="A1:AT108"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:46">
@@ -16925,6 +16952,286 @@
         <v>1.7</v>
       </c>
     </row>
+    <row r="107" spans="1:46">
+      <c r="A107" t="s">
+        <v>46</v>
+      </c>
+      <c r="B107" t="s">
+        <v>552</v>
+      </c>
+      <c r="C107" t="s">
+        <v>579</v>
+      </c>
+      <c r="D107">
+        <v>84042</v>
+      </c>
+      <c r="E107">
+        <v>25616</v>
+      </c>
+      <c r="F107" t="b">
+        <v>1</v>
+      </c>
+      <c r="G107" t="s">
+        <v>580</v>
+      </c>
+      <c r="H107" t="s">
+        <v>568</v>
+      </c>
+      <c r="I107">
+        <v>7230</v>
+      </c>
+      <c r="J107" t="s">
+        <v>581</v>
+      </c>
+      <c r="K107">
+        <v>4468</v>
+      </c>
+      <c r="L107">
+        <v>1361.85</v>
+      </c>
+      <c r="M107">
+        <v>140.9</v>
+      </c>
+      <c r="N107">
+        <v>87.55</v>
+      </c>
+      <c r="O107">
+        <v>39.20616666666667</v>
+      </c>
+      <c r="P107">
+        <v>-102.48566666666666</v>
+      </c>
+      <c r="Q107">
+        <v>5214</v>
+      </c>
+      <c r="R107">
+        <v>1589.23</v>
+      </c>
+      <c r="S107">
+        <v>39.608</v>
+      </c>
+      <c r="T107">
+        <v>-104.04216666666666</v>
+      </c>
+      <c r="U107" t="s">
+        <v>156</v>
+      </c>
+      <c r="V107">
+        <v>83849</v>
+      </c>
+      <c r="W107">
+        <v>25557.18</v>
+      </c>
+      <c r="X107">
+        <v>251</v>
+      </c>
+      <c r="Y107" t="s">
+        <v>53</v>
+      </c>
+      <c r="Z107">
+        <v>12</v>
+      </c>
+      <c r="AA107">
+        <v>3.66</v>
+      </c>
+      <c r="AB107">
+        <v>0.77</v>
+      </c>
+      <c r="AC107">
+        <v>1.7</v>
+      </c>
+      <c r="AD107">
+        <v>140.9</v>
+      </c>
+      <c r="AE107">
+        <v>87.55</v>
+      </c>
+      <c r="AF107" t="s">
+        <v>582</v>
+      </c>
+      <c r="AG107">
+        <v>3</v>
+      </c>
+      <c r="AH107">
+        <v>6.61</v>
+      </c>
+      <c r="AI107">
+        <v>4.75</v>
+      </c>
+      <c r="AJ107">
+        <v>10.48</v>
+      </c>
+      <c r="AK107">
+        <v>1.53</v>
+      </c>
+      <c r="AL107">
+        <v>3.38</v>
+      </c>
+      <c r="AM107">
+        <v>10.06</v>
+      </c>
+      <c r="AN107">
+        <v>22.17</v>
+      </c>
+      <c r="AO107">
+        <v>9.07</v>
+      </c>
+      <c r="AP107">
+        <v>19.99</v>
+      </c>
+      <c r="AQ107">
+        <v>7.06</v>
+      </c>
+      <c r="AR107">
+        <v>15.56</v>
+      </c>
+      <c r="AS107">
+        <v>0.77</v>
+      </c>
+      <c r="AT107">
+        <v>1.7</v>
+      </c>
+    </row>
+    <row r="108" spans="1:46">
+      <c r="A108" t="s">
+        <v>46</v>
+      </c>
+      <c r="B108" t="s">
+        <v>583</v>
+      </c>
+      <c r="C108" t="s">
+        <v>579</v>
+      </c>
+      <c r="D108">
+        <v>96668</v>
+      </c>
+      <c r="E108">
+        <v>29464.41</v>
+      </c>
+      <c r="F108" t="b">
+        <v>1</v>
+      </c>
+      <c r="G108" t="s">
+        <v>584</v>
+      </c>
+      <c r="H108" t="s">
+        <v>585</v>
+      </c>
+      <c r="I108">
+        <v>8370</v>
+      </c>
+      <c r="J108" t="s">
+        <v>586</v>
+      </c>
+      <c r="K108">
+        <v>5253</v>
+      </c>
+      <c r="L108">
+        <v>1601.11</v>
+      </c>
+      <c r="M108">
+        <v>166.37</v>
+      </c>
+      <c r="N108">
+        <v>103.38</v>
+      </c>
+      <c r="O108">
+        <v>39.13243333333334</v>
+      </c>
+      <c r="P108">
+        <v>-102.20588333333332</v>
+      </c>
+      <c r="Q108">
+        <v>5224</v>
+      </c>
+      <c r="R108">
+        <v>1592.28</v>
+      </c>
+      <c r="S108">
+        <v>39.6082</v>
+      </c>
+      <c r="T108">
+        <v>-104.0423</v>
+      </c>
+      <c r="U108" t="s">
+        <v>156</v>
+      </c>
+      <c r="V108">
+        <v>96417</v>
+      </c>
+      <c r="W108">
+        <v>29387.9</v>
+      </c>
+      <c r="X108">
+        <v>800</v>
+      </c>
+      <c r="Y108" t="s">
+        <v>53</v>
+      </c>
+      <c r="Z108">
+        <v>12</v>
+      </c>
+      <c r="AA108">
+        <v>3.66</v>
+      </c>
+      <c r="AB108">
+        <v>0.82</v>
+      </c>
+      <c r="AC108">
+        <v>1.81</v>
+      </c>
+      <c r="AD108">
+        <v>166.37</v>
+      </c>
+      <c r="AE108">
+        <v>103.38</v>
+      </c>
+      <c r="AF108" t="s">
+        <v>587</v>
+      </c>
+      <c r="AG108">
+        <v>3</v>
+      </c>
+      <c r="AH108">
+        <v>6.61</v>
+      </c>
+      <c r="AI108">
+        <v>5.06</v>
+      </c>
+      <c r="AJ108">
+        <v>11.15</v>
+      </c>
+      <c r="AK108">
+        <v>2.2</v>
+      </c>
+      <c r="AL108">
+        <v>4.84</v>
+      </c>
+      <c r="AM108">
+        <v>11.07</v>
+      </c>
+      <c r="AN108">
+        <v>24.41</v>
+      </c>
+      <c r="AO108">
+        <v>10.29</v>
+      </c>
+      <c r="AP108">
+        <v>22.68</v>
+      </c>
+      <c r="AQ108">
+        <v>8.07</v>
+      </c>
+      <c r="AR108">
+        <v>17.8</v>
+      </c>
+      <c r="AS108">
+        <v>0.82</v>
+      </c>
+      <c r="AT108">
+        <v>1.81</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Updates for flights 398, 399, & 400
</commit_message>
<xml_diff>
--- a/www/flightdata/xlsx/flights_metadata.xlsx
+++ b/www/flightdata/xlsx/flights_metadata.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1009" uniqueCount="588">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1036" uniqueCount="602">
   <si>
     <t>balloonsize</t>
   </si>
@@ -1778,6 +1778,48 @@
   </si>
   <si>
     <t>[{"altitude_ft":36584.0,"altitude_m":11150.8,"transition":"high_to_low"}]</t>
+  </si>
+  <si>
+    <t>["KC0D-2","K0SCC-13"]</t>
+  </si>
+  <si>
+    <t>2026-05-02</t>
+  </si>
+  <si>
+    <t>EOSS-398</t>
+  </si>
+  <si>
+    <t>1hrs 48mins 30secs</t>
+  </si>
+  <si>
+    <t>293</t>
+  </si>
+  <si>
+    <t>[{"altitude_ft":52824.0,"altitude_m":16100.76,"transition":"high_to_low"}]</t>
+  </si>
+  <si>
+    <t>["KC0D-3","AE0SS-3"]</t>
+  </si>
+  <si>
+    <t>EOSS-399</t>
+  </si>
+  <si>
+    <t>[{"altitude_ft":46553.0,"altitude_m":14189.35,"transition":"high_to_low"}]</t>
+  </si>
+  <si>
+    <t>["KC0D-14","AE0SS-4","K0SCC-14"]</t>
+  </si>
+  <si>
+    <t>EOSS-400</t>
+  </si>
+  <si>
+    <t>2hrs 13mins 0secs</t>
+  </si>
+  <si>
+    <t>316</t>
+  </si>
+  <si>
+    <t>[{"altitude_ft":41058.0,"altitude_m":12514.48,"transition":"high_to_low"}]</t>
   </si>
 </sst>
 </file>
@@ -2109,7 +2151,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AT108"/>
+  <dimension ref="A1:AT111"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:46">
@@ -17232,6 +17274,426 @@
         <v>1.81</v>
       </c>
     </row>
+    <row r="109" spans="1:46">
+      <c r="A109" t="s">
+        <v>62</v>
+      </c>
+      <c r="B109" t="s">
+        <v>588</v>
+      </c>
+      <c r="C109" t="s">
+        <v>589</v>
+      </c>
+      <c r="D109">
+        <v>89253</v>
+      </c>
+      <c r="E109">
+        <v>27204.31</v>
+      </c>
+      <c r="F109" t="b">
+        <v>1</v>
+      </c>
+      <c r="G109" t="s">
+        <v>590</v>
+      </c>
+      <c r="H109" t="s">
+        <v>591</v>
+      </c>
+      <c r="I109">
+        <v>6510</v>
+      </c>
+      <c r="J109" t="s">
+        <v>592</v>
+      </c>
+      <c r="K109">
+        <v>7525</v>
+      </c>
+      <c r="L109">
+        <v>2293.62</v>
+      </c>
+      <c r="M109">
+        <v>54.17</v>
+      </c>
+      <c r="N109">
+        <v>33.66</v>
+      </c>
+      <c r="O109">
+        <v>39.27166666666667</v>
+      </c>
+      <c r="P109">
+        <v>-103.58533333333334</v>
+      </c>
+      <c r="Q109">
+        <v>5222</v>
+      </c>
+      <c r="R109">
+        <v>1591.67</v>
+      </c>
+      <c r="S109">
+        <v>39.608</v>
+      </c>
+      <c r="T109">
+        <v>-104.04216666666666</v>
+      </c>
+      <c r="U109" t="s">
+        <v>118</v>
+      </c>
+      <c r="V109">
+        <v>89063</v>
+      </c>
+      <c r="W109">
+        <v>27146.4</v>
+      </c>
+      <c r="X109">
+        <v>417</v>
+      </c>
+      <c r="Y109" t="s">
+        <v>53</v>
+      </c>
+      <c r="Z109">
+        <v>12</v>
+      </c>
+      <c r="AA109">
+        <v>3.66</v>
+      </c>
+      <c r="AB109">
+        <v>0.77</v>
+      </c>
+      <c r="AC109">
+        <v>1.7</v>
+      </c>
+      <c r="AD109">
+        <v>54.17</v>
+      </c>
+      <c r="AE109">
+        <v>33.66</v>
+      </c>
+      <c r="AF109" t="s">
+        <v>593</v>
+      </c>
+      <c r="AG109">
+        <v>1.5</v>
+      </c>
+      <c r="AH109">
+        <v>3.31</v>
+      </c>
+      <c r="AI109">
+        <v>3.7</v>
+      </c>
+      <c r="AJ109">
+        <v>8.16</v>
+      </c>
+      <c r="AK109">
+        <v>1.61</v>
+      </c>
+      <c r="AL109">
+        <v>3.54</v>
+      </c>
+      <c r="AM109">
+        <v>7.57</v>
+      </c>
+      <c r="AN109">
+        <v>16.7</v>
+      </c>
+      <c r="AO109">
+        <v>8.35</v>
+      </c>
+      <c r="AP109">
+        <v>18.4</v>
+      </c>
+      <c r="AQ109">
+        <v>6.07</v>
+      </c>
+      <c r="AR109">
+        <v>13.39</v>
+      </c>
+      <c r="AS109">
+        <v>0.77</v>
+      </c>
+      <c r="AT109">
+        <v>1.7</v>
+      </c>
+    </row>
+    <row r="110" spans="1:46">
+      <c r="A110" t="s">
+        <v>62</v>
+      </c>
+      <c r="B110" t="s">
+        <v>594</v>
+      </c>
+      <c r="C110" t="s">
+        <v>589</v>
+      </c>
+      <c r="D110">
+        <v>87335</v>
+      </c>
+      <c r="E110">
+        <v>26619.71</v>
+      </c>
+      <c r="F110" t="b">
+        <v>1</v>
+      </c>
+      <c r="G110" t="s">
+        <v>595</v>
+      </c>
+      <c r="H110" t="s">
+        <v>286</v>
+      </c>
+      <c r="I110">
+        <v>6390</v>
+      </c>
+      <c r="J110" t="s">
+        <v>258</v>
+      </c>
+      <c r="K110">
+        <v>8061</v>
+      </c>
+      <c r="L110">
+        <v>2456.99</v>
+      </c>
+      <c r="M110">
+        <v>54.36</v>
+      </c>
+      <c r="N110">
+        <v>33.78</v>
+      </c>
+      <c r="O110">
+        <v>39.261833333333335</v>
+      </c>
+      <c r="P110">
+        <v>-103.5945</v>
+      </c>
+      <c r="Q110">
+        <v>5202</v>
+      </c>
+      <c r="R110">
+        <v>1585.57</v>
+      </c>
+      <c r="S110">
+        <v>39.608</v>
+      </c>
+      <c r="T110">
+        <v>-104.04216666666666</v>
+      </c>
+      <c r="U110" t="s">
+        <v>118</v>
+      </c>
+      <c r="V110">
+        <v>87123</v>
+      </c>
+      <c r="W110">
+        <v>26555.09</v>
+      </c>
+      <c r="X110">
+        <v>409</v>
+      </c>
+      <c r="Y110" t="s">
+        <v>53</v>
+      </c>
+      <c r="Z110">
+        <v>12</v>
+      </c>
+      <c r="AA110">
+        <v>3.66</v>
+      </c>
+      <c r="AB110">
+        <v>0.82</v>
+      </c>
+      <c r="AC110">
+        <v>1.81</v>
+      </c>
+      <c r="AD110">
+        <v>54.36</v>
+      </c>
+      <c r="AE110">
+        <v>33.78</v>
+      </c>
+      <c r="AF110" t="s">
+        <v>596</v>
+      </c>
+      <c r="AG110">
+        <v>1.5</v>
+      </c>
+      <c r="AH110">
+        <v>3.31</v>
+      </c>
+      <c r="AI110">
+        <v>3.6</v>
+      </c>
+      <c r="AJ110">
+        <v>7.94</v>
+      </c>
+      <c r="AK110">
+        <v>1.77</v>
+      </c>
+      <c r="AL110">
+        <v>3.9</v>
+      </c>
+      <c r="AM110">
+        <v>7.69</v>
+      </c>
+      <c r="AN110">
+        <v>16.95</v>
+      </c>
+      <c r="AO110">
+        <v>8.5</v>
+      </c>
+      <c r="AP110">
+        <v>18.73</v>
+      </c>
+      <c r="AQ110">
+        <v>6.19</v>
+      </c>
+      <c r="AR110">
+        <v>13.65</v>
+      </c>
+      <c r="AS110">
+        <v>0.82</v>
+      </c>
+      <c r="AT110">
+        <v>1.81</v>
+      </c>
+    </row>
+    <row r="111" spans="1:46">
+      <c r="A111" t="s">
+        <v>46</v>
+      </c>
+      <c r="B111" t="s">
+        <v>597</v>
+      </c>
+      <c r="C111" t="s">
+        <v>589</v>
+      </c>
+      <c r="D111">
+        <v>107271</v>
+      </c>
+      <c r="E111">
+        <v>32696.2</v>
+      </c>
+      <c r="F111" t="b">
+        <v>1</v>
+      </c>
+      <c r="G111" t="s">
+        <v>598</v>
+      </c>
+      <c r="H111" t="s">
+        <v>599</v>
+      </c>
+      <c r="I111">
+        <v>7980</v>
+      </c>
+      <c r="J111" t="s">
+        <v>600</v>
+      </c>
+      <c r="K111">
+        <v>9380</v>
+      </c>
+      <c r="L111">
+        <v>2859.02</v>
+      </c>
+      <c r="M111">
+        <v>65.13</v>
+      </c>
+      <c r="N111">
+        <v>40.47</v>
+      </c>
+      <c r="O111">
+        <v>39.30533333333333</v>
+      </c>
+      <c r="P111">
+        <v>-103.392</v>
+      </c>
+      <c r="Q111">
+        <v>5206</v>
+      </c>
+      <c r="R111">
+        <v>1586.79</v>
+      </c>
+      <c r="S111">
+        <v>39.608</v>
+      </c>
+      <c r="T111">
+        <v>-104.04216666666666</v>
+      </c>
+      <c r="U111" t="s">
+        <v>156</v>
+      </c>
+      <c r="V111">
+        <v>107044</v>
+      </c>
+      <c r="W111">
+        <v>32627.01</v>
+      </c>
+      <c r="X111">
+        <v>705</v>
+      </c>
+      <c r="Y111" t="s">
+        <v>53</v>
+      </c>
+      <c r="Z111">
+        <v>12</v>
+      </c>
+      <c r="AA111">
+        <v>3.66</v>
+      </c>
+      <c r="AB111">
+        <v>0.77</v>
+      </c>
+      <c r="AC111">
+        <v>1.7</v>
+      </c>
+      <c r="AD111">
+        <v>65.13</v>
+      </c>
+      <c r="AE111">
+        <v>40.47</v>
+      </c>
+      <c r="AF111" t="s">
+        <v>601</v>
+      </c>
+      <c r="AG111">
+        <v>3</v>
+      </c>
+      <c r="AH111">
+        <v>6.61</v>
+      </c>
+      <c r="AI111">
+        <v>3</v>
+      </c>
+      <c r="AJ111">
+        <v>6.61</v>
+      </c>
+      <c r="AK111">
+        <v>2.08</v>
+      </c>
+      <c r="AL111">
+        <v>4.59</v>
+      </c>
+      <c r="AM111">
+        <v>8.85</v>
+      </c>
+      <c r="AN111">
+        <v>19.51</v>
+      </c>
+      <c r="AO111">
+        <v>7.62</v>
+      </c>
+      <c r="AP111">
+        <v>16.8</v>
+      </c>
+      <c r="AQ111">
+        <v>5.85</v>
+      </c>
+      <c r="AR111">
+        <v>12.9</v>
+      </c>
+      <c r="AS111">
+        <v>0.77</v>
+      </c>
+      <c r="AT111">
+        <v>1.7</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Updates for flights EOSS-401 and EOSS-402
</commit_message>
<xml_diff>
--- a/www/flightdata/xlsx/flights_metadata.xlsx
+++ b/www/flightdata/xlsx/flights_metadata.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1036" uniqueCount="602">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1054" uniqueCount="610">
   <si>
     <t>balloonsize</t>
   </si>
@@ -1820,6 +1820,30 @@
   </si>
   <si>
     <t>[{"altitude_ft":41058.0,"altitude_m":12514.48,"transition":"high_to_low"}]</t>
+  </si>
+  <si>
+    <t>2026-05-09</t>
+  </si>
+  <si>
+    <t>EOSS-401</t>
+  </si>
+  <si>
+    <t>321</t>
+  </si>
+  <si>
+    <t>[{"altitude_ft":41732.0,"altitude_m":12719.91,"transition":"high_to_low"}]</t>
+  </si>
+  <si>
+    <t>EOSS-402</t>
+  </si>
+  <si>
+    <t>2hrs 0mins 0secs</t>
+  </si>
+  <si>
+    <t>319</t>
+  </si>
+  <si>
+    <t>[{"altitude_ft":40554.0,"altitude_m":12360.86,"transition":"high_to_low"}]</t>
   </si>
 </sst>
 </file>
@@ -2151,7 +2175,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AT111"/>
+  <dimension ref="A1:AT113"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:46">
@@ -17694,6 +17718,286 @@
         <v>1.7</v>
       </c>
     </row>
+    <row r="112" spans="1:46">
+      <c r="A112" t="s">
+        <v>46</v>
+      </c>
+      <c r="B112" t="s">
+        <v>588</v>
+      </c>
+      <c r="C112" t="s">
+        <v>602</v>
+      </c>
+      <c r="D112">
+        <v>75129</v>
+      </c>
+      <c r="E112">
+        <v>22899.32</v>
+      </c>
+      <c r="F112" t="b">
+        <v>1</v>
+      </c>
+      <c r="G112" t="s">
+        <v>603</v>
+      </c>
+      <c r="H112" t="s">
+        <v>443</v>
+      </c>
+      <c r="I112">
+        <v>6900</v>
+      </c>
+      <c r="J112" t="s">
+        <v>604</v>
+      </c>
+      <c r="K112">
+        <v>4692</v>
+      </c>
+      <c r="L112">
+        <v>1430.12</v>
+      </c>
+      <c r="M112">
+        <v>97.61</v>
+      </c>
+      <c r="N112">
+        <v>60.65</v>
+      </c>
+      <c r="O112">
+        <v>39.30148333333333</v>
+      </c>
+      <c r="P112">
+        <v>-102.97625</v>
+      </c>
+      <c r="Q112">
+        <v>5214</v>
+      </c>
+      <c r="R112">
+        <v>1589.23</v>
+      </c>
+      <c r="S112">
+        <v>39.608183333333336</v>
+      </c>
+      <c r="T112">
+        <v>-104.04228333333332</v>
+      </c>
+      <c r="U112" t="s">
+        <v>156</v>
+      </c>
+      <c r="V112">
+        <v>75055</v>
+      </c>
+      <c r="W112">
+        <v>22876.76</v>
+      </c>
+      <c r="X112">
+        <v>447</v>
+      </c>
+      <c r="Y112" t="s">
+        <v>53</v>
+      </c>
+      <c r="Z112">
+        <v>12</v>
+      </c>
+      <c r="AA112">
+        <v>3.66</v>
+      </c>
+      <c r="AB112">
+        <v>0.77</v>
+      </c>
+      <c r="AC112">
+        <v>1.7</v>
+      </c>
+      <c r="AD112">
+        <v>97.61</v>
+      </c>
+      <c r="AE112">
+        <v>60.65</v>
+      </c>
+      <c r="AF112" t="s">
+        <v>605</v>
+      </c>
+      <c r="AG112">
+        <v>3</v>
+      </c>
+      <c r="AH112">
+        <v>6.61</v>
+      </c>
+      <c r="AI112">
+        <v>3.32</v>
+      </c>
+      <c r="AJ112">
+        <v>7.31</v>
+      </c>
+      <c r="AK112">
+        <v>1.89</v>
+      </c>
+      <c r="AL112">
+        <v>4.16</v>
+      </c>
+      <c r="AM112">
+        <v>8.98</v>
+      </c>
+      <c r="AN112">
+        <v>19.79</v>
+      </c>
+      <c r="AO112">
+        <v>7.77</v>
+      </c>
+      <c r="AP112">
+        <v>17.13</v>
+      </c>
+      <c r="AQ112">
+        <v>5.97</v>
+      </c>
+      <c r="AR112">
+        <v>13.17</v>
+      </c>
+      <c r="AS112">
+        <v>0.77</v>
+      </c>
+      <c r="AT112">
+        <v>1.7</v>
+      </c>
+    </row>
+    <row r="113" spans="1:46">
+      <c r="A113" t="s">
+        <v>46</v>
+      </c>
+      <c r="B113" t="s">
+        <v>594</v>
+      </c>
+      <c r="C113" t="s">
+        <v>602</v>
+      </c>
+      <c r="D113">
+        <v>72643</v>
+      </c>
+      <c r="E113">
+        <v>22141.59</v>
+      </c>
+      <c r="F113" t="b">
+        <v>1</v>
+      </c>
+      <c r="G113" t="s">
+        <v>606</v>
+      </c>
+      <c r="H113" t="s">
+        <v>607</v>
+      </c>
+      <c r="I113">
+        <v>7200</v>
+      </c>
+      <c r="J113" t="s">
+        <v>608</v>
+      </c>
+      <c r="K113">
+        <v>4824</v>
+      </c>
+      <c r="L113">
+        <v>1470.36</v>
+      </c>
+      <c r="M113">
+        <v>104.12</v>
+      </c>
+      <c r="N113">
+        <v>64.7</v>
+      </c>
+      <c r="O113">
+        <v>39.2435</v>
+      </c>
+      <c r="P113">
+        <v>-102.92466666666668</v>
+      </c>
+      <c r="Q113">
+        <v>5216</v>
+      </c>
+      <c r="R113">
+        <v>1589.84</v>
+      </c>
+      <c r="S113">
+        <v>39.608</v>
+      </c>
+      <c r="T113">
+        <v>-104.04216666666666</v>
+      </c>
+      <c r="U113" t="s">
+        <v>156</v>
+      </c>
+      <c r="V113">
+        <v>72570</v>
+      </c>
+      <c r="W113">
+        <v>22119.34</v>
+      </c>
+      <c r="X113">
+        <v>445</v>
+      </c>
+      <c r="Y113" t="s">
+        <v>53</v>
+      </c>
+      <c r="Z113">
+        <v>12</v>
+      </c>
+      <c r="AA113">
+        <v>3.66</v>
+      </c>
+      <c r="AB113">
+        <v>0.77</v>
+      </c>
+      <c r="AC113">
+        <v>1.7</v>
+      </c>
+      <c r="AD113">
+        <v>104.12</v>
+      </c>
+      <c r="AE113">
+        <v>64.7</v>
+      </c>
+      <c r="AF113" t="s">
+        <v>609</v>
+      </c>
+      <c r="AG113">
+        <v>3</v>
+      </c>
+      <c r="AH113">
+        <v>6.61</v>
+      </c>
+      <c r="AI113">
+        <v>3.45</v>
+      </c>
+      <c r="AJ113">
+        <v>7.61</v>
+      </c>
+      <c r="AK113">
+        <v>1.7</v>
+      </c>
+      <c r="AL113">
+        <v>3.74</v>
+      </c>
+      <c r="AM113">
+        <v>8.92</v>
+      </c>
+      <c r="AN113">
+        <v>19.66</v>
+      </c>
+      <c r="AO113">
+        <v>7.7</v>
+      </c>
+      <c r="AP113">
+        <v>16.97</v>
+      </c>
+      <c r="AQ113">
+        <v>5.91</v>
+      </c>
+      <c r="AR113">
+        <v>13.04</v>
+      </c>
+      <c r="AS113">
+        <v>0.77</v>
+      </c>
+      <c r="AT113">
+        <v>1.7</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Update for flight EOSS-405
</commit_message>
<xml_diff>
--- a/www/flightdata/xlsx/flights_metadata.xlsx
+++ b/www/flightdata/xlsx/flights_metadata.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1072" uniqueCount="621">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1081" uniqueCount="625">
   <si>
     <t>balloonsize</t>
   </si>
@@ -1877,6 +1877,18 @@
   </si>
   <si>
     <t>[{"altitude_ft":56609.0,"altitude_m":17254.42,"transition":"high_to_low"}]</t>
+  </si>
+  <si>
+    <t>2026-08-22</t>
+  </si>
+  <si>
+    <t>EOSS-405</t>
+  </si>
+  <si>
+    <t>342</t>
+  </si>
+  <si>
+    <t>[{"altitude_ft":10113.0,"altitude_m":3082.44,"transition":"low_to_high"},{"altitude_ft":61473.0,"altitude_m":18736.97,"transition":"high_to_low"}]</t>
   </si>
 </sst>
 </file>
@@ -2208,7 +2220,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AT115"/>
+  <dimension ref="A1:AT116"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:46">
@@ -18311,6 +18323,146 @@
         <v>1.7</v>
       </c>
     </row>
+    <row r="116" spans="1:46">
+      <c r="A116" t="s">
+        <v>46</v>
+      </c>
+      <c r="B116" t="s">
+        <v>588</v>
+      </c>
+      <c r="C116" t="s">
+        <v>621</v>
+      </c>
+      <c r="D116">
+        <v>107526</v>
+      </c>
+      <c r="E116">
+        <v>32773.92</v>
+      </c>
+      <c r="F116" t="b">
+        <v>1</v>
+      </c>
+      <c r="G116" t="s">
+        <v>622</v>
+      </c>
+      <c r="H116" t="s">
+        <v>272</v>
+      </c>
+      <c r="I116">
+        <v>7470</v>
+      </c>
+      <c r="J116" t="s">
+        <v>623</v>
+      </c>
+      <c r="K116">
+        <v>5467</v>
+      </c>
+      <c r="L116">
+        <v>1666.34</v>
+      </c>
+      <c r="M116">
+        <v>27.02</v>
+      </c>
+      <c r="N116">
+        <v>16.79</v>
+      </c>
+      <c r="O116">
+        <v>38.993833333333335</v>
+      </c>
+      <c r="P116">
+        <v>-103.72301666666668</v>
+      </c>
+      <c r="Q116">
+        <v>5408</v>
+      </c>
+      <c r="R116">
+        <v>1648.36</v>
+      </c>
+      <c r="S116">
+        <v>39.23613333333333</v>
+      </c>
+      <c r="T116">
+        <v>-103.69696666666668</v>
+      </c>
+      <c r="U116" t="s">
+        <v>156</v>
+      </c>
+      <c r="V116">
+        <v>106755</v>
+      </c>
+      <c r="W116">
+        <v>32538.92</v>
+      </c>
+      <c r="X116">
+        <v>425</v>
+      </c>
+      <c r="Y116" t="s">
+        <v>53</v>
+      </c>
+      <c r="Z116">
+        <v>12</v>
+      </c>
+      <c r="AA116">
+        <v>3.66</v>
+      </c>
+      <c r="AB116">
+        <v>0.77</v>
+      </c>
+      <c r="AC116">
+        <v>1.7</v>
+      </c>
+      <c r="AD116">
+        <v>27.02</v>
+      </c>
+      <c r="AE116">
+        <v>16.79</v>
+      </c>
+      <c r="AF116" t="s">
+        <v>624</v>
+      </c>
+      <c r="AG116">
+        <v>3</v>
+      </c>
+      <c r="AH116">
+        <v>6.61</v>
+      </c>
+      <c r="AI116">
+        <v>3.72</v>
+      </c>
+      <c r="AJ116">
+        <v>8.21</v>
+      </c>
+      <c r="AK116">
+        <v>2.08</v>
+      </c>
+      <c r="AL116">
+        <v>4.58</v>
+      </c>
+      <c r="AM116">
+        <v>9.57</v>
+      </c>
+      <c r="AN116">
+        <v>21.1</v>
+      </c>
+      <c r="AO116">
+        <v>8.48</v>
+      </c>
+      <c r="AP116">
+        <v>18.7</v>
+      </c>
+      <c r="AQ116">
+        <v>6.57</v>
+      </c>
+      <c r="AR116">
+        <v>14.48</v>
+      </c>
+      <c r="AS116">
+        <v>0.77</v>
+      </c>
+      <c r="AT116">
+        <v>1.7</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>